<commit_message>
Atualiza painel (2026-10-02 11:05 UTC)
</commit_message>
<xml_diff>
--- a/dados/status_atual.xlsx
+++ b/dados/status_atual.xlsx
@@ -452,7 +452,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>96.5</v>
+        <v>97</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -463,7 +463,7 @@
         <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>310</v>
+        <v>318</v>
       </c>
     </row>
     <row r="3">
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>80.8</v>
+        <v>80.2</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -484,7 +484,7 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>295</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>70.8</v>
+        <v>71.5</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -505,7 +505,7 @@
         <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="5">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>59.5</v>
+        <v>60.6</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -526,7 +526,7 @@
         <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>266</v>
+        <v>276</v>
       </c>
     </row>
     <row r="6">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>44.4</v>
+        <v>44.6</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -547,7 +547,7 @@
         <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>289</v>
+        <v>297</v>
       </c>
     </row>
     <row r="7">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>25.6</v>
+        <v>26.7</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -568,7 +568,7 @@
         <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>276</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -644,19 +644,19 @@
         </is>
       </c>
       <c r="D2" t="n">
+        <v>67</v>
+      </c>
+      <c r="E2" t="n">
         <v>65</v>
       </c>
-      <c r="E2" t="n">
-        <v>62</v>
-      </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>95.40000000000001</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3">
@@ -676,10 +676,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E3" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
@@ -708,10 +708,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E4" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F4" t="n">
         <v>5</v>
@@ -720,7 +720,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>94.59999999999999</v>
+        <v>94.7</v>
       </c>
     </row>
     <row r="5">
@@ -740,10 +740,10 @@
         </is>
       </c>
       <c r="D5" t="n">
+        <v>74</v>
+      </c>
+      <c r="E5" t="n">
         <v>72</v>
-      </c>
-      <c r="E5" t="n">
-        <v>70</v>
       </c>
       <c r="F5" t="n">
         <v>2</v>
@@ -752,7 +752,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>97.2</v>
+        <v>97.3</v>
       </c>
     </row>
     <row r="6">
@@ -772,19 +772,19 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E6" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>86.40000000000001</v>
+        <v>87.7</v>
       </c>
     </row>
     <row r="7">
@@ -804,19 +804,19 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E7" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>84.59999999999999</v>
+        <v>82.7</v>
       </c>
     </row>
     <row r="8">
@@ -836,10 +836,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="E8" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F8" t="n">
         <v>23</v>
@@ -848,7 +848,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>75</v>
+        <v>74.2</v>
       </c>
     </row>
     <row r="9">
@@ -868,10 +868,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E9" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F9" t="n">
         <v>15</v>
@@ -880,7 +880,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>77.3</v>
+        <v>76.2</v>
       </c>
     </row>
     <row r="10">
@@ -900,10 +900,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E10" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F10" t="n">
         <v>18</v>
@@ -912,7 +912,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>66</v>
+        <v>67.3</v>
       </c>
     </row>
     <row r="11">
@@ -932,19 +932,19 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E11" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F11" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>56.5</v>
+        <v>56.9</v>
       </c>
     </row>
     <row r="12">
@@ -964,19 +964,19 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E12" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F12" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>56.8</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="13">
@@ -996,19 +996,19 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E13" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F13" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>58.7</v>
+        <v>58.5</v>
       </c>
     </row>
     <row r="14">
@@ -1028,10 +1028,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E14" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F14" t="n">
         <v>34</v>
@@ -1040,7 +1040,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>41.4</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="15">
@@ -1060,19 +1060,19 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E15" t="n">
         <v>38</v>
       </c>
       <c r="F15" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>49.4</v>
+        <v>48.1</v>
       </c>
     </row>
     <row r="16">
@@ -1092,10 +1092,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E16" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F16" t="n">
         <v>53</v>
@@ -1104,7 +1104,7 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>39.1</v>
+        <v>40.4</v>
       </c>
     </row>
     <row r="17">
@@ -1124,19 +1124,19 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E17" t="n">
         <v>32</v>
       </c>
       <c r="F17" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>47.8</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="18">
@@ -1156,19 +1156,19 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E18" t="n">
         <v>17</v>
       </c>
       <c r="F18" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>28.8</v>
+        <v>30.4</v>
       </c>
     </row>
     <row r="19">
@@ -1188,19 +1188,19 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E19" t="n">
         <v>14</v>
       </c>
       <c r="F19" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>19.4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20">
@@ -1220,19 +1220,19 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
       </c>
       <c r="F20" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>25.9</v>
+        <v>26.9</v>
       </c>
     </row>
     <row r="21">
@@ -1252,19 +1252,19 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E21" t="n">
         <v>18</v>
       </c>
       <c r="F21" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>28.1</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="22">
@@ -1287,16 +1287,16 @@
         <v>58</v>
       </c>
       <c r="E22" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F22" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>72.40000000000001</v>
+        <v>74.09999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -1348,19 +1348,19 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E24" t="n">
         <v>59</v>
       </c>
       <c r="F24" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>69.40000000000001</v>
+        <v>70.2</v>
       </c>
     </row>
     <row r="25">
@@ -2062,7 +2062,7 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>-10.92</v>
+        <v>13.06</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -2111,7 +2111,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>1294.9</v>
+        <v>1318.88</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -2215,7 +2215,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>-9.470000000000001</v>
+        <v>14.51</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -2374,7 +2374,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>1415.38</v>
+        <v>1439.36</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Em avaliação</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2468,18 +2468,24 @@
           <t>2026-09-27T00:39:16.889629+00:00</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-10-02T10:22:55.333927+00:00</t>
+        </is>
+      </c>
       <c r="G20" t="n">
         <v>67.06999999999999</v>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>129.73</v>
+      </c>
+      <c r="I20" t="n">
+        <v>196.8</v>
+      </c>
       <c r="J20" t="b">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>173.53</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -2559,7 +2565,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Associado</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2572,18 +2578,24 @@
           <t>2026-09-29T02:51:50.216902+00:00</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-10-02T08:27:18.009434+00:00</t>
+        </is>
+      </c>
       <c r="G22" t="n">
         <v>55.58</v>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>77.59</v>
+      </c>
+      <c r="I22" t="n">
+        <v>133.17</v>
+      </c>
       <c r="J22" t="b">
-        <v>0</v>
-      </c>
-      <c r="K22" t="n">
-        <v>111.82</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -2796,7 +2808,7 @@
         <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>720.39</v>
+        <v>744.37</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -3175,7 +3187,7 @@
         <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>229.27</v>
+        <v>253.24</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -3224,7 +3236,7 @@
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>1389.2</v>
+        <v>1413.18</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -3438,7 +3450,7 @@
         <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>0.82</v>
+        <v>24.8</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -3597,7 +3609,7 @@
         <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>50.72</v>
+        <v>74.7</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -3678,45 +3690,39 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Em avaliação</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2026-08-09T22:25:40.706812+00:00</t>
+          <t>2026-10-05T23:28:41.696937+00:00</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-08-10T04:28:17.183184+00:00</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>2026-08-11T16:04:22.771041+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-06T05:31:18.173309+00:00</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="n">
         <v>6.04</v>
       </c>
-      <c r="H43" t="n">
-        <v>35.6</v>
-      </c>
-      <c r="I43" t="n">
-        <v>41.65</v>
-      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
       <c r="J43" t="b">
-        <v>1</v>
-      </c>
-      <c r="K43" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K43" t="n">
+        <v>-84.39</v>
+      </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2026-S32</t>
+          <t>2026-S41</t>
         </is>
       </c>
     </row>
@@ -3756,7 +3762,7 @@
         <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>625.76</v>
+        <v>649.73</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
@@ -3970,7 +3976,7 @@
         <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>286.71</v>
+        <v>310.68</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -4459,7 +4465,7 @@
         <v>0</v>
       </c>
       <c r="K57" t="n">
-        <v>-66.86</v>
+        <v>-42.88</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
@@ -4508,7 +4514,7 @@
         <v>0</v>
       </c>
       <c r="K58" t="n">
-        <v>1113.3</v>
+        <v>1137.27</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
@@ -4667,7 +4673,7 @@
         <v>0</v>
       </c>
       <c r="K61" t="n">
-        <v>906.51</v>
+        <v>930.49</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -4716,7 +4722,7 @@
         <v>0</v>
       </c>
       <c r="K62" t="n">
-        <v>1367.36</v>
+        <v>1391.34</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -4875,7 +4881,7 @@
         <v>0</v>
       </c>
       <c r="K65" t="n">
-        <v>135.68</v>
+        <v>159.65</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
@@ -4901,7 +4907,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Associado</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -4914,18 +4920,24 @@
           <t>2026-09-28T10:34:41.222399+00:00</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2026-10-02T07:53:44.672077+00:00</t>
+        </is>
+      </c>
       <c r="G66" t="n">
         <v>16.77</v>
       </c>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
+      <c r="H66" t="n">
+        <v>93.31999999999999</v>
+      </c>
+      <c r="I66" t="n">
+        <v>110.08</v>
+      </c>
       <c r="J66" t="b">
-        <v>0</v>
-      </c>
-      <c r="K66" t="n">
-        <v>89.3</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -5028,7 +5040,7 @@
         <v>0</v>
       </c>
       <c r="K68" t="n">
-        <v>123.82</v>
+        <v>147.8</v>
       </c>
       <c r="L68" t="inlineStr">
         <is>
@@ -5077,7 +5089,7 @@
         <v>0</v>
       </c>
       <c r="K69" t="n">
-        <v>29.61</v>
+        <v>53.59</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -5103,7 +5115,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -5116,18 +5128,24 @@
           <t>2026-09-27T07:23:39.065444+00:00</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>2026-10-01T22:33:59.238483+00:00</t>
+        </is>
+      </c>
       <c r="G70" t="n">
         <v>35.16</v>
       </c>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
+      <c r="H70" t="n">
+        <v>111.17</v>
+      </c>
+      <c r="I70" t="n">
+        <v>146.33</v>
+      </c>
       <c r="J70" t="b">
-        <v>0</v>
-      </c>
-      <c r="K70" t="n">
-        <v>134.88</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -5285,7 +5303,7 @@
         <v>0</v>
       </c>
       <c r="K73" t="n">
-        <v>92.95999999999999</v>
+        <v>116.93</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -5389,7 +5407,7 @@
         <v>0</v>
       </c>
       <c r="K75" t="n">
-        <v>-92.38</v>
+        <v>-68.41</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -5548,7 +5566,7 @@
         <v>0</v>
       </c>
       <c r="K78" t="n">
-        <v>94.81</v>
+        <v>118.78</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
@@ -5872,7 +5890,7 @@
         <v>0</v>
       </c>
       <c r="K84" t="n">
-        <v>165.78</v>
+        <v>189.76</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -6636,7 +6654,7 @@
         <v>0</v>
       </c>
       <c r="K98" t="n">
-        <v>348.22</v>
+        <v>372.2</v>
       </c>
       <c r="L98" t="inlineStr">
         <is>
@@ -6722,12 +6740,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>2026-09-17T18:36:22.389810+00:00</t>
+          <t>2026-10-02T18:36:22.389810+00:00</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>2026-09-18T05:14:05.999230+00:00</t>
+          <t>2026-10-03T05:14:05.999230+00:00</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -6740,16 +6758,16 @@
         <v>0</v>
       </c>
       <c r="K100" t="n">
-        <v>328.5</v>
+        <v>-7.52</v>
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>2026-S38</t>
+          <t>2026-S40</t>
         </is>
       </c>
     </row>
@@ -6789,7 +6807,7 @@
         <v>0</v>
       </c>
       <c r="K101" t="n">
-        <v>85.23</v>
+        <v>109.21</v>
       </c>
       <c r="L101" t="inlineStr">
         <is>
@@ -6893,7 +6911,7 @@
         <v>0</v>
       </c>
       <c r="K103" t="n">
-        <v>-1.63</v>
+        <v>22.35</v>
       </c>
       <c r="L103" t="inlineStr">
         <is>
@@ -6997,7 +7015,7 @@
         <v>0</v>
       </c>
       <c r="K105" t="n">
-        <v>391.64</v>
+        <v>415.62</v>
       </c>
       <c r="L105" t="inlineStr">
         <is>
@@ -7046,7 +7064,7 @@
         <v>0</v>
       </c>
       <c r="K106" t="n">
-        <v>46.89</v>
+        <v>70.86</v>
       </c>
       <c r="L106" t="inlineStr">
         <is>
@@ -7370,7 +7388,7 @@
         <v>0</v>
       </c>
       <c r="K112" t="n">
-        <v>679.96</v>
+        <v>703.9400000000001</v>
       </c>
       <c r="L112" t="inlineStr">
         <is>
@@ -7804,7 +7822,7 @@
         <v>0</v>
       </c>
       <c r="K120" t="n">
-        <v>30</v>
+        <v>53.98</v>
       </c>
       <c r="L120" t="inlineStr">
         <is>
@@ -8128,7 +8146,7 @@
         <v>0</v>
       </c>
       <c r="K126" t="n">
-        <v>-9.289999999999999</v>
+        <v>14.69</v>
       </c>
       <c r="L126" t="inlineStr">
         <is>
@@ -8177,7 +8195,7 @@
         <v>0</v>
       </c>
       <c r="K127" t="n">
-        <v>-53.55</v>
+        <v>-29.57</v>
       </c>
       <c r="L127" t="inlineStr">
         <is>
@@ -8258,7 +8276,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Em avaliação</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -8271,18 +8289,24 @@
           <t>2026-09-30T19:43:39.259439+00:00</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr"/>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>2026-10-02T00:10:12.391049+00:00</t>
+        </is>
+      </c>
       <c r="G129" t="n">
         <v>7.73</v>
       </c>
-      <c r="H129" t="inlineStr"/>
-      <c r="I129" t="inlineStr"/>
+      <c r="H129" t="n">
+        <v>28.44</v>
+      </c>
+      <c r="I129" t="n">
+        <v>36.18</v>
+      </c>
       <c r="J129" t="b">
-        <v>0</v>
-      </c>
-      <c r="K129" t="n">
-        <v>23.12</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K129" t="inlineStr"/>
       <c r="L129" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -8385,7 +8409,7 @@
         <v>0</v>
       </c>
       <c r="K131" t="n">
-        <v>384.26</v>
+        <v>408.24</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
@@ -8819,7 +8843,7 @@
         <v>0</v>
       </c>
       <c r="K139" t="n">
-        <v>709.41</v>
+        <v>733.39</v>
       </c>
       <c r="L139" t="inlineStr">
         <is>
@@ -8868,7 +8892,7 @@
         <v>0</v>
       </c>
       <c r="K140" t="n">
-        <v>414.92</v>
+        <v>438.9</v>
       </c>
       <c r="L140" t="inlineStr">
         <is>
@@ -8917,7 +8941,7 @@
         <v>0</v>
       </c>
       <c r="K141" t="n">
-        <v>1356.36</v>
+        <v>1380.34</v>
       </c>
       <c r="L141" t="inlineStr">
         <is>
@@ -9131,7 +9155,7 @@
         <v>0</v>
       </c>
       <c r="K145" t="n">
-        <v>1071.2</v>
+        <v>1095.18</v>
       </c>
       <c r="L145" t="inlineStr">
         <is>
@@ -9290,7 +9314,7 @@
         <v>0</v>
       </c>
       <c r="K148" t="n">
-        <v>478.12</v>
+        <v>502.1</v>
       </c>
       <c r="L148" t="inlineStr">
         <is>
@@ -9339,7 +9363,7 @@
         <v>0</v>
       </c>
       <c r="K149" t="n">
-        <v>486.96</v>
+        <v>510.94</v>
       </c>
       <c r="L149" t="inlineStr">
         <is>
@@ -9365,7 +9389,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -9378,18 +9402,24 @@
           <t>2026-09-28T23:59:44.282440+00:00</t>
         </is>
       </c>
-      <c r="F150" t="inlineStr"/>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>2026-10-02T01:19:43.435676+00:00</t>
+        </is>
+      </c>
       <c r="G150" t="n">
         <v>42.96</v>
       </c>
-      <c r="H150" t="inlineStr"/>
-      <c r="I150" t="inlineStr"/>
+      <c r="H150" t="n">
+        <v>73.33</v>
+      </c>
+      <c r="I150" t="n">
+        <v>116.29</v>
+      </c>
       <c r="J150" t="b">
-        <v>0</v>
-      </c>
-      <c r="K150" t="n">
-        <v>102.07</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -9602,7 +9632,7 @@
         <v>0</v>
       </c>
       <c r="K154" t="n">
-        <v>334.8</v>
+        <v>358.78</v>
       </c>
       <c r="L154" t="inlineStr">
         <is>
@@ -10123,52 +10153,46 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Pendente</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>2026-08-06T13:14:21.949146+00:00</t>
+          <t>2026-10-06T01:40:46.286073+00:00</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>2026-08-07T09:28:41.720911+00:00</t>
-        </is>
-      </c>
-      <c r="F164" t="inlineStr">
-        <is>
-          <t>2026-08-08T07:48:09.271745+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-07T17:05:11.725115+00:00</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr"/>
       <c r="G164" t="n">
-        <v>20.24</v>
-      </c>
-      <c r="H164" t="n">
-        <v>22.32</v>
-      </c>
-      <c r="I164" t="n">
-        <v>42.56</v>
-      </c>
+        <v>39.41</v>
+      </c>
+      <c r="H164" t="inlineStr"/>
+      <c r="I164" t="inlineStr"/>
       <c r="J164" t="b">
-        <v>1</v>
-      </c>
-      <c r="K164" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K164" t="n">
+        <v>-86.59</v>
+      </c>
       <c r="L164" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>2026-S32</t>
+          <t>2026-S41</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Bravo Casa</t>
+          <t>Delta Sports</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -10178,51 +10202,57 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Associado</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>2026-09-29T02:04:17.345631+00:00</t>
+          <t>2026-08-10T01:55:04.685035+00:00</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>2026-09-30T04:08:23.850223+00:00</t>
-        </is>
-      </c>
-      <c r="F165" t="inlineStr"/>
+          <t>2026-08-11T07:52:46.764366+00:00</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>2026-08-17T02:21:21.693144+00:00</t>
+        </is>
+      </c>
       <c r="G165" t="n">
-        <v>26.07</v>
-      </c>
-      <c r="H165" t="inlineStr"/>
-      <c r="I165" t="inlineStr"/>
+        <v>29.96</v>
+      </c>
+      <c r="H165" t="n">
+        <v>138.48</v>
+      </c>
+      <c r="I165" t="n">
+        <v>168.44</v>
+      </c>
       <c r="J165" t="b">
-        <v>0</v>
-      </c>
-      <c r="K165" t="n">
-        <v>57.04</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K165" t="inlineStr"/>
       <c r="L165" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>2026-S40</t>
+          <t>2026-S33</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Bravo Casa</t>
+          <t>Fluxo Denim</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>PO-10256</t>
+          <t>PO-10257</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -10232,27 +10262,27 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>2026-08-26T22:26:51.613292+00:00</t>
+          <t>2026-08-20T02:12:17.791952+00:00</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>2026-08-28T06:07:25.113334+00:00</t>
+          <t>2026-08-21T01:15:41.529315+00:00</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>2026-08-31T02:27:00.205867+00:00</t>
+          <t>2026-08-23T02:32:57.687537+00:00</t>
         </is>
       </c>
       <c r="G166" t="n">
-        <v>31.68</v>
+        <v>23.06</v>
       </c>
       <c r="H166" t="n">
-        <v>68.33</v>
+        <v>49.29</v>
       </c>
       <c r="I166" t="n">
-        <v>100</v>
+        <v>72.34</v>
       </c>
       <c r="J166" t="b">
         <v>1</v>
@@ -10265,19 +10295,19 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>2026-S35</t>
+          <t>2026-S34</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Cedro Kids</t>
+          <t>Delta Sports</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>PO-10257</t>
+          <t>PO-10258</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -10287,27 +10317,27 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>2026-08-16T18:21:05.974360+00:00</t>
+          <t>2026-09-18T11:21:05.974360+00:00</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>2026-08-17T10:34:55.170763+00:00</t>
+          <t>2026-09-19T06:30:00.067414+00:00</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>2026-08-20T06:29:59.460695+00:00</t>
+          <t>2026-09-22T14:37:43.412998+00:00</t>
         </is>
       </c>
       <c r="G167" t="n">
-        <v>16.23</v>
+        <v>19.15</v>
       </c>
       <c r="H167" t="n">
-        <v>67.92</v>
+        <v>80.13</v>
       </c>
       <c r="I167" t="n">
-        <v>84.15000000000001</v>
+        <v>99.28</v>
       </c>
       <c r="J167" t="b">
         <v>1</v>
@@ -10315,12 +10345,12 @@
       <c r="K167" t="inlineStr"/>
       <c r="L167" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>2026-S33</t>
+          <t>2026-S38</t>
         </is>
       </c>
     </row>
@@ -10332,7 +10362,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>PO-10258</t>
+          <t>PO-10259</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -10387,7 +10417,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>PO-10259</t>
+          <t>PO-10260</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -10415,7 +10445,7 @@
         <v>0</v>
       </c>
       <c r="K169" t="n">
-        <v>-53.36</v>
+        <v>-29.39</v>
       </c>
       <c r="L169" t="inlineStr">
         <is>
@@ -10436,7 +10466,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>PO-10260</t>
+          <t>PO-10261</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -10491,7 +10521,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>PO-10261</t>
+          <t>PO-10262</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -10546,7 +10576,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>PO-10262</t>
+          <t>PO-10263</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -10601,7 +10631,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>PO-10264</t>
+          <t>PO-10265</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -10656,7 +10686,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>PO-10265</t>
+          <t>PO-10266</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -10711,7 +10741,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>PO-10266</t>
+          <t>PO-10267</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -10766,7 +10796,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>PO-10267</t>
+          <t>PO-10268</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -10821,7 +10851,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>PO-10268</t>
+          <t>PO-10269</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -10849,7 +10879,7 @@
         <v>0</v>
       </c>
       <c r="K177" t="n">
-        <v>207.94</v>
+        <v>231.91</v>
       </c>
       <c r="L177" t="inlineStr">
         <is>
@@ -10870,12 +10900,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>PO-10269</t>
+          <t>PO-10270</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -10888,18 +10918,24 @@
           <t>2026-09-29T21:51:15.180525+00:00</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr"/>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>2026-10-01T23:18:34.610039+00:00</t>
+        </is>
+      </c>
       <c r="G178" t="n">
         <v>21.26</v>
       </c>
-      <c r="H178" t="inlineStr"/>
-      <c r="I178" t="inlineStr"/>
+      <c r="H178" t="n">
+        <v>49.46</v>
+      </c>
+      <c r="I178" t="n">
+        <v>70.72</v>
+      </c>
       <c r="J178" t="b">
-        <v>0</v>
-      </c>
-      <c r="K178" t="n">
-        <v>58.52</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K178" t="inlineStr"/>
       <c r="L178" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -10919,7 +10955,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>PO-10271</t>
+          <t>PO-10272</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -10974,7 +11010,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>PO-10272</t>
+          <t>PO-10273</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -11029,50 +11065,44 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>PO-10273</t>
+          <t>PO-10274</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Pendente</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>2026-08-31T04:02:57.860442+00:00</t>
+          <t>2026-10-07T02:02:57.860442+00:00</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>2026-08-31T22:00:30.459000+00:00</t>
-        </is>
-      </c>
-      <c r="F181" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:42:55.394632+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-07T20:00:30.459000+00:00</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr"/>
       <c r="G181" t="n">
         <v>17.96</v>
       </c>
-      <c r="H181" t="n">
-        <v>11.71</v>
-      </c>
-      <c r="I181" t="n">
-        <v>29.67</v>
-      </c>
+      <c r="H181" t="inlineStr"/>
+      <c r="I181" t="inlineStr"/>
       <c r="J181" t="b">
-        <v>1</v>
-      </c>
-      <c r="K181" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K181" t="n">
+        <v>-110.96</v>
+      </c>
       <c r="L181" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>2026-S36</t>
+          <t>2026-S41</t>
         </is>
       </c>
     </row>
@@ -11084,7 +11114,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>PO-10274</t>
+          <t>PO-10275</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -11139,7 +11169,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>PO-10276</t>
+          <t>PO-10277</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -11194,7 +11224,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>PO-10277</t>
+          <t>PO-10278</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -11249,7 +11279,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>PO-10280</t>
+          <t>PO-10281</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -11277,7 +11307,7 @@
         <v>0</v>
       </c>
       <c r="K185" t="n">
-        <v>446.12</v>
+        <v>470.1</v>
       </c>
       <c r="L185" t="inlineStr">
         <is>
@@ -11298,7 +11328,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>PO-10281</t>
+          <t>PO-10282</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -11353,7 +11383,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>PO-10282</t>
+          <t>PO-10283</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -11381,7 +11411,7 @@
         <v>0</v>
       </c>
       <c r="K187" t="n">
-        <v>1018.68</v>
+        <v>1042.66</v>
       </c>
       <c r="L187" t="inlineStr">
         <is>
@@ -11402,7 +11432,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>PO-10285</t>
+          <t>PO-10286</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -11457,7 +11487,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>PO-10286</t>
+          <t>PO-10287</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -11485,7 +11515,7 @@
         <v>0</v>
       </c>
       <c r="K189" t="n">
-        <v>-35.64</v>
+        <v>-11.66</v>
       </c>
       <c r="L189" t="inlineStr">
         <is>
@@ -11506,7 +11536,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>PO-10287</t>
+          <t>PO-10288</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -11561,7 +11591,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>PO-10288</t>
+          <t>PO-10289</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -11589,7 +11619,7 @@
         <v>0</v>
       </c>
       <c r="K191" t="n">
-        <v>580.85</v>
+        <v>604.8200000000001</v>
       </c>
       <c r="L191" t="inlineStr">
         <is>
@@ -11610,7 +11640,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>PO-10291</t>
+          <t>PO-10292</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -11665,7 +11695,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>PO-10292</t>
+          <t>PO-10293</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -11720,7 +11750,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>PO-10295</t>
+          <t>PO-10296</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -11775,7 +11805,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>PO-10296</t>
+          <t>PO-10297</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -11830,7 +11860,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>PO-10297</t>
+          <t>PO-10298</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -11858,7 +11888,7 @@
         <v>0</v>
       </c>
       <c r="K196" t="n">
-        <v>-0.47</v>
+        <v>23.51</v>
       </c>
       <c r="L196" t="inlineStr">
         <is>
@@ -11879,7 +11909,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>PO-10299</t>
+          <t>PO-10300</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -11934,7 +11964,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>PO-10300</t>
+          <t>PO-10301</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -11989,7 +12019,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>PO-10301</t>
+          <t>PO-10302</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -12017,7 +12047,7 @@
         <v>0</v>
       </c>
       <c r="K199" t="n">
-        <v>388.35</v>
+        <v>412.32</v>
       </c>
       <c r="L199" t="inlineStr">
         <is>
@@ -12038,7 +12068,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>PO-10302</t>
+          <t>PO-10303</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -12093,7 +12123,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>PO-10303</t>
+          <t>PO-10304</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -12148,7 +12178,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>PO-10304</t>
+          <t>PO-10305</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -12203,7 +12233,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>PO-10305</t>
+          <t>PO-10306</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -12231,7 +12261,7 @@
         <v>0</v>
       </c>
       <c r="K203" t="n">
-        <v>1429.91</v>
+        <v>1453.89</v>
       </c>
       <c r="L203" t="inlineStr">
         <is>
@@ -12252,91 +12282,91 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>PO-10306</t>
+          <t>PO-10307</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Associado</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>2026-09-14T18:54:12.862542+00:00</t>
+          <t>2026-10-05T07:42:11.435008+00:00</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>2026-09-15T07:59:32.068592+00:00</t>
-        </is>
-      </c>
-      <c r="F204" t="inlineStr">
-        <is>
-          <t>2026-09-18T03:47:33.625700+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-06T10:05:17.414086+00:00</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr"/>
       <c r="G204" t="n">
-        <v>13.09</v>
-      </c>
-      <c r="H204" t="n">
-        <v>67.8</v>
-      </c>
-      <c r="I204" t="n">
-        <v>80.89</v>
-      </c>
+        <v>26.38</v>
+      </c>
+      <c r="H204" t="inlineStr"/>
+      <c r="I204" t="inlineStr"/>
       <c r="J204" t="b">
-        <v>1</v>
-      </c>
-      <c r="K204" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K204" t="n">
+        <v>-68.62</v>
+      </c>
       <c r="L204" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>2026-S38</t>
+          <t>2026-S41</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Eterna Beleza</t>
+          <t>Cedro Kids</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>PO-10307</t>
+          <t>PO-10308</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Associado</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>2026-09-04T15:59:31.160800+00:00</t>
+          <t>2026-09-06T21:39:59.170057+00:00</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>2026-09-07T20:39:13.537141+00:00</t>
-        </is>
-      </c>
-      <c r="F205" t="inlineStr"/>
+          <t>2026-09-07T14:28:57.504614+00:00</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>2026-09-11T15:42:21.924110+00:00</t>
+        </is>
+      </c>
       <c r="G205" t="n">
-        <v>76.66</v>
-      </c>
-      <c r="H205" t="inlineStr"/>
-      <c r="I205" t="inlineStr"/>
+        <v>16.82</v>
+      </c>
+      <c r="H205" t="n">
+        <v>97.22</v>
+      </c>
+      <c r="I205" t="n">
+        <v>114.04</v>
+      </c>
       <c r="J205" t="b">
-        <v>0</v>
-      </c>
-      <c r="K205" t="n">
-        <v>643.12</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K205" t="inlineStr"/>
       <c r="L205" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -12356,7 +12386,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>PO-10308</t>
+          <t>PO-10309</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -12366,17 +12396,17 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>2026-09-20T10:54:56.507681+00:00</t>
+          <t>2026-09-18T03:19:24.896933+00:00</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>2026-09-21T17:25:30.100123+00:00</t>
+          <t>2026-09-19T09:49:58.489375+00:00</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>2026-09-23T01:33:09.789206+00:00</t>
+          <t>2026-09-20T17:57:38.178458+00:00</t>
         </is>
       </c>
       <c r="G206" t="n">
@@ -12411,7 +12441,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>PO-10309</t>
+          <t>PO-10310</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -12466,7 +12496,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>PO-10311</t>
+          <t>PO-10312</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -12521,7 +12551,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>PO-10312</t>
+          <t>PO-10313</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -12576,7 +12606,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>PO-10313</t>
+          <t>PO-10314</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -12631,7 +12661,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>PO-10314</t>
+          <t>PO-10315</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -12659,7 +12689,7 @@
         <v>0</v>
       </c>
       <c r="K211" t="n">
-        <v>673.46</v>
+        <v>697.4400000000001</v>
       </c>
       <c r="L211" t="inlineStr">
         <is>
@@ -12680,7 +12710,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>PO-10315</t>
+          <t>PO-10316</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -12708,7 +12738,7 @@
         <v>0</v>
       </c>
       <c r="K212" t="n">
-        <v>474.89</v>
+        <v>498.87</v>
       </c>
       <c r="L212" t="inlineStr">
         <is>
@@ -12729,7 +12759,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>PO-10316</t>
+          <t>PO-10317</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -12784,7 +12814,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>PO-10317</t>
+          <t>PO-10318</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -12839,7 +12869,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>PO-10318</t>
+          <t>PO-10319</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -12867,7 +12897,7 @@
         <v>0</v>
       </c>
       <c r="K215" t="n">
-        <v>337.01</v>
+        <v>360.99</v>
       </c>
       <c r="L215" t="inlineStr">
         <is>
@@ -12888,7 +12918,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>PO-10320</t>
+          <t>PO-10321</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -12943,7 +12973,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>PO-10321</t>
+          <t>PO-10322</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -12998,7 +13028,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>PO-10322</t>
+          <t>PO-10323</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -13053,7 +13083,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>PO-10323</t>
+          <t>PO-10324</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -13108,7 +13138,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>PO-10324</t>
+          <t>PO-10325</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -13136,7 +13166,7 @@
         <v>0</v>
       </c>
       <c r="K220" t="n">
-        <v>753.11</v>
+        <v>777.09</v>
       </c>
       <c r="L220" t="inlineStr">
         <is>
@@ -13157,7 +13187,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>PO-10326</t>
+          <t>PO-10327</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -13185,7 +13215,7 @@
         <v>0</v>
       </c>
       <c r="K221" t="n">
-        <v>303.36</v>
+        <v>327.34</v>
       </c>
       <c r="L221" t="inlineStr">
         <is>
@@ -13206,7 +13236,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>PO-10328</t>
+          <t>PO-10329</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -13261,7 +13291,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>PO-10329</t>
+          <t>PO-10330</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -13316,7 +13346,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>PO-10330</t>
+          <t>PO-10331</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -13371,7 +13401,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>PO-10331</t>
+          <t>PO-10332</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -13426,7 +13456,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>PO-10334</t>
+          <t>PO-10335</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -13481,7 +13511,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>PO-10335</t>
+          <t>PO-10336</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -13536,7 +13566,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>PO-10336</t>
+          <t>PO-10337</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -13564,7 +13594,7 @@
         <v>0</v>
       </c>
       <c r="K228" t="n">
-        <v>1262.34</v>
+        <v>1286.31</v>
       </c>
       <c r="L228" t="inlineStr">
         <is>
@@ -13585,7 +13615,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>PO-10337</t>
+          <t>PO-10338</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -13640,7 +13670,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>PO-10339</t>
+          <t>PO-10340</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -13695,7 +13725,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>PO-10341</t>
+          <t>PO-10342</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -13750,7 +13780,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>PO-10343</t>
+          <t>PO-10344</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -13778,7 +13808,7 @@
         <v>0</v>
       </c>
       <c r="K232" t="n">
-        <v>230.54</v>
+        <v>254.51</v>
       </c>
       <c r="L232" t="inlineStr">
         <is>
@@ -13799,7 +13829,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>PO-10345</t>
+          <t>PO-10346</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -13827,7 +13857,7 @@
         <v>0</v>
       </c>
       <c r="K233" t="n">
-        <v>995.25</v>
+        <v>1019.23</v>
       </c>
       <c r="L233" t="inlineStr">
         <is>
@@ -13848,7 +13878,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>PO-10346</t>
+          <t>PO-10347</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -13903,7 +13933,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>PO-10347</t>
+          <t>PO-10348</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -13931,7 +13961,7 @@
         <v>0</v>
       </c>
       <c r="K235" t="n">
-        <v>856.12</v>
+        <v>880.1</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -13952,7 +13982,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>PO-10348</t>
+          <t>PO-10349</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -14007,7 +14037,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>PO-10350</t>
+          <t>PO-10351</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -14062,7 +14092,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>PO-10351</t>
+          <t>PO-10352</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -14117,7 +14147,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>PO-10352</t>
+          <t>PO-10353</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -14145,7 +14175,7 @@
         <v>0</v>
       </c>
       <c r="K239" t="n">
-        <v>87.09</v>
+        <v>111.06</v>
       </c>
       <c r="L239" t="inlineStr">
         <is>
@@ -14166,7 +14196,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>PO-10355</t>
+          <t>PO-10356</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -14221,7 +14251,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>PO-10356</t>
+          <t>PO-10357</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -14276,7 +14306,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>PO-10357</t>
+          <t>PO-10358</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -14331,7 +14361,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>PO-10359</t>
+          <t>PO-10360</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -14386,7 +14416,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>PO-10360</t>
+          <t>PO-10361</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -14441,7 +14471,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>PO-10361</t>
+          <t>PO-10362</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -14469,7 +14499,7 @@
         <v>0</v>
       </c>
       <c r="K245" t="n">
-        <v>504.54</v>
+        <v>528.52</v>
       </c>
       <c r="L245" t="inlineStr">
         <is>
@@ -14490,7 +14520,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>PO-10362</t>
+          <t>PO-10363</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -14545,7 +14575,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>PO-10365</t>
+          <t>PO-10366</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -14573,7 +14603,7 @@
         <v>0</v>
       </c>
       <c r="K247" t="n">
-        <v>983.58</v>
+        <v>1007.56</v>
       </c>
       <c r="L247" t="inlineStr">
         <is>
@@ -14594,12 +14624,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>PO-10366</t>
+          <t>PO-10367</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -14612,18 +14642,24 @@
           <t>2026-09-29T13:21:38.418091+00:00</t>
         </is>
       </c>
-      <c r="F248" t="inlineStr"/>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>2026-10-01T20:23:49.036603+00:00</t>
+        </is>
+      </c>
       <c r="G248" t="n">
         <v>30.97</v>
       </c>
-      <c r="H248" t="inlineStr"/>
-      <c r="I248" t="inlineStr"/>
+      <c r="H248" t="n">
+        <v>55.04</v>
+      </c>
+      <c r="I248" t="n">
+        <v>86.01000000000001</v>
+      </c>
       <c r="J248" t="b">
-        <v>0</v>
-      </c>
-      <c r="K248" t="n">
-        <v>76.72</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K248" t="inlineStr"/>
       <c r="L248" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -14643,7 +14679,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>PO-10370</t>
+          <t>PO-10371</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -14698,7 +14734,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>PO-10372</t>
+          <t>PO-10373</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -14753,7 +14789,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>PO-10373</t>
+          <t>PO-10374</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -14808,7 +14844,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>PO-10374</t>
+          <t>PO-10375</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -14863,7 +14899,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>PO-10375</t>
+          <t>PO-10376</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -14918,7 +14954,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>PO-10377</t>
+          <t>PO-10378</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -14973,50 +15009,44 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>PO-10378</t>
+          <t>PO-10379</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Em avaliação</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>2026-09-11T02:14:31.207658+00:00</t>
+          <t>2026-10-05T18:36:22.873224+00:00</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>2026-09-14T09:42:56.059057+00:00</t>
-        </is>
-      </c>
-      <c r="F255" t="inlineStr">
-        <is>
-          <t>2026-09-14T18:02:17.331216+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-08T18:32:08.951469+00:00</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr"/>
       <c r="G255" t="n">
-        <v>79.47</v>
-      </c>
-      <c r="H255" t="n">
-        <v>8.32</v>
-      </c>
-      <c r="I255" t="n">
-        <v>87.8</v>
-      </c>
+        <v>71.93000000000001</v>
+      </c>
+      <c r="H255" t="inlineStr"/>
+      <c r="I255" t="inlineStr"/>
       <c r="J255" t="b">
-        <v>1</v>
-      </c>
-      <c r="K255" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K255" t="n">
+        <v>-79.52</v>
+      </c>
       <c r="L255" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>2026-S37</t>
+          <t>2026-S41</t>
         </is>
       </c>
     </row>
@@ -15028,7 +15058,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>PO-10379</t>
+          <t>PO-10380</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -15038,27 +15068,27 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>2026-08-25T05:24:55.068175+00:00</t>
+          <t>2026-08-11T18:22:57.141658+00:00</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2026-08-26T12:00:56.568902+00:00</t>
+          <t>2026-08-12T05:28:15.465215+00:00</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>2026-08-27T22:30:46.179863+00:00</t>
+          <t>2026-08-15T12:44:42.023063+00:00</t>
         </is>
       </c>
       <c r="G256" t="n">
-        <v>30.6</v>
+        <v>11.09</v>
       </c>
       <c r="H256" t="n">
-        <v>34.5</v>
+        <v>79.27</v>
       </c>
       <c r="I256" t="n">
-        <v>65.09999999999999</v>
+        <v>90.36</v>
       </c>
       <c r="J256" t="b">
         <v>1</v>
@@ -15071,19 +15101,19 @@
       </c>
       <c r="M256" t="inlineStr">
         <is>
-          <t>2026-S35</t>
+          <t>2026-S33</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Fluxo Denim</t>
+          <t>Alpha Moda</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>PO-10380</t>
+          <t>PO-10381</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -15093,27 +15123,27 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>2026-08-17T11:08:27.132700+00:00</t>
+          <t>2026-09-20T06:59:16.386510+00:00</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>2026-08-17T17:53:34.280401+00:00</t>
+          <t>2026-09-20T11:56:25.990140+00:00</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>2026-08-20T03:36:03.912050+00:00</t>
+          <t>2026-09-22T06:16:13.001242+00:00</t>
         </is>
       </c>
       <c r="G257" t="n">
-        <v>6.75</v>
+        <v>4.95</v>
       </c>
       <c r="H257" t="n">
-        <v>57.71</v>
+        <v>42.33</v>
       </c>
       <c r="I257" t="n">
-        <v>64.45999999999999</v>
+        <v>47.28</v>
       </c>
       <c r="J257" t="b">
         <v>1</v>
@@ -15121,12 +15151,12 @@
       <c r="K257" t="inlineStr"/>
       <c r="L257" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="M257" t="inlineStr">
         <is>
-          <t>2026-S34</t>
+          <t>2026-S38</t>
         </is>
       </c>
     </row>
@@ -15138,7 +15168,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>PO-10384</t>
+          <t>PO-10385</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -15193,7 +15223,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>PO-10385</t>
+          <t>PO-10386</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -15221,7 +15251,7 @@
         <v>0</v>
       </c>
       <c r="K259" t="n">
-        <v>355.72</v>
+        <v>379.69</v>
       </c>
       <c r="L259" t="inlineStr">
         <is>
@@ -15242,7 +15272,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>PO-10386</t>
+          <t>PO-10387</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -15297,7 +15327,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>PO-10388</t>
+          <t>PO-10389</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -15352,7 +15382,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>PO-10389</t>
+          <t>PO-10390</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -15407,7 +15437,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>PO-10390</t>
+          <t>PO-10391</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -15462,7 +15492,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>PO-10391</t>
+          <t>PO-10392</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -15517,7 +15547,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>PO-10393</t>
+          <t>PO-10394</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -15572,7 +15602,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>PO-10394</t>
+          <t>PO-10395</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -15627,7 +15657,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>PO-10395</t>
+          <t>PO-10396</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -15682,7 +15712,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>PO-10397</t>
+          <t>PO-10398</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -15737,7 +15767,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>PO-10398</t>
+          <t>PO-10399</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -15792,7 +15822,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>PO-10399</t>
+          <t>PO-10400</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -15847,57 +15877,51 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>PO-10400</t>
+          <t>PO-10401</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Em avaliação</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>2026-08-20T07:35:51.118964+00:00</t>
+          <t>2026-10-05T03:54:26.066066+00:00</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>2026-08-21T06:25:59.213884+00:00</t>
-        </is>
-      </c>
-      <c r="F271" t="inlineStr">
-        <is>
-          <t>2026-08-25T00:56:44.642840+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-07T01:40:09.879960+00:00</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr"/>
       <c r="G271" t="n">
-        <v>22.84</v>
-      </c>
-      <c r="H271" t="n">
-        <v>90.51000000000001</v>
-      </c>
-      <c r="I271" t="n">
-        <v>113.35</v>
-      </c>
+        <v>45.76</v>
+      </c>
+      <c r="H271" t="inlineStr"/>
+      <c r="I271" t="inlineStr"/>
       <c r="J271" t="b">
-        <v>1</v>
-      </c>
-      <c r="K271" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K271" t="n">
+        <v>-64.81999999999999</v>
+      </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="M271" t="inlineStr">
         <is>
-          <t>2026-S34</t>
+          <t>2026-S41</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Alpha Moda</t>
+          <t>Cedro Kids</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -15912,27 +15936,27 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>2026-08-28T11:13:11.819187+00:00</t>
+          <t>2026-08-17T06:30:13.021464+00:00</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>2026-08-30T04:11:39.547603+00:00</t>
+          <t>2026-08-18T07:16:03.603156+00:00</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>2026-08-31T11:32:08.683302+00:00</t>
+          <t>2026-08-22T12:11:51.999925+00:00</t>
         </is>
       </c>
       <c r="G272" t="n">
-        <v>40.97</v>
+        <v>24.76</v>
       </c>
       <c r="H272" t="n">
-        <v>31.34</v>
+        <v>100.93</v>
       </c>
       <c r="I272" t="n">
-        <v>72.31999999999999</v>
+        <v>125.69</v>
       </c>
       <c r="J272" t="b">
         <v>1</v>
@@ -15945,19 +15969,19 @@
       </c>
       <c r="M272" t="inlineStr">
         <is>
-          <t>2026-S35</t>
+          <t>2026-S34</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Eterna Beleza</t>
+          <t>Alpha Moda</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>PO-10403</t>
+          <t>PO-10404</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -15967,27 +15991,27 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>2026-08-21T01:03:32.678636+00:00</t>
+          <t>2026-08-06T18:56:03.575526+00:00</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>2026-08-22T13:41:22.932773+00:00</t>
+          <t>2026-08-07T11:27:28.406997+00:00</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>2026-08-24T10:03:51.214342+00:00</t>
+          <t>2026-08-08T12:56:16.822739+00:00</t>
         </is>
       </c>
       <c r="G273" t="n">
-        <v>36.63</v>
+        <v>16.52</v>
       </c>
       <c r="H273" t="n">
-        <v>44.37</v>
+        <v>25.48</v>
       </c>
       <c r="I273" t="n">
-        <v>81.01000000000001</v>
+        <v>42</v>
       </c>
       <c r="J273" t="b">
         <v>1</v>
@@ -16000,7 +16024,7 @@
       </c>
       <c r="M273" t="inlineStr">
         <is>
-          <t>2026-S34</t>
+          <t>2026-S32</t>
         </is>
       </c>
     </row>
@@ -16012,7 +16036,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>PO-10407</t>
+          <t>PO-10408</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -16067,7 +16091,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>PO-10409</t>
+          <t>PO-10410</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -16122,7 +16146,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>PO-10410</t>
+          <t>PO-10411</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -16177,7 +16201,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>PO-10411</t>
+          <t>PO-10412</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -16205,7 +16229,7 @@
         <v>0</v>
       </c>
       <c r="K277" t="n">
-        <v>1127.34</v>
+        <v>1151.32</v>
       </c>
       <c r="L277" t="inlineStr">
         <is>
@@ -16226,7 +16250,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>PO-10412</t>
+          <t>PO-10413</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -16254,7 +16278,7 @@
         <v>0</v>
       </c>
       <c r="K278" t="n">
-        <v>1358.6</v>
+        <v>1382.57</v>
       </c>
       <c r="L278" t="inlineStr">
         <is>
@@ -16275,7 +16299,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>PO-10415</t>
+          <t>PO-10416</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -16303,7 +16327,7 @@
         <v>0</v>
       </c>
       <c r="K279" t="n">
-        <v>434.51</v>
+        <v>458.49</v>
       </c>
       <c r="L279" t="inlineStr">
         <is>
@@ -16324,7 +16348,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>PO-10416</t>
+          <t>PO-10417</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -16352,7 +16376,7 @@
         <v>0</v>
       </c>
       <c r="K280" t="n">
-        <v>170.56</v>
+        <v>194.54</v>
       </c>
       <c r="L280" t="inlineStr">
         <is>
@@ -16373,7 +16397,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>PO-10418</t>
+          <t>PO-10419</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -16401,7 +16425,7 @@
         <v>0</v>
       </c>
       <c r="K281" t="n">
-        <v>12.64</v>
+        <v>36.61</v>
       </c>
       <c r="L281" t="inlineStr">
         <is>
@@ -16422,7 +16446,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>PO-10419</t>
+          <t>PO-10420</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -16450,7 +16474,7 @@
         <v>0</v>
       </c>
       <c r="K282" t="n">
-        <v>914.15</v>
+        <v>938.13</v>
       </c>
       <c r="L282" t="inlineStr">
         <is>
@@ -16471,7 +16495,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>PO-10420</t>
+          <t>PO-10421</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -16481,12 +16505,12 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>2026-09-06T14:23:05.319402+00:00</t>
+          <t>2026-10-05T15:23:05.319402+00:00</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>2026-09-08T11:11:41.342139+00:00</t>
+          <t>2026-10-07T12:11:41.342139+00:00</t>
         </is>
       </c>
       <c r="F283" t="inlineStr"/>
@@ -16499,16 +16523,16 @@
         <v>0</v>
       </c>
       <c r="K283" t="n">
-        <v>596.73</v>
+        <v>-76.3</v>
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>2026-S36</t>
+          <t>2026-S41</t>
         </is>
       </c>
     </row>
@@ -16520,7 +16544,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>PO-10421</t>
+          <t>PO-10422</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -16575,7 +16599,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>PO-10422</t>
+          <t>PO-10423</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -16630,7 +16654,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>PO-10423</t>
+          <t>PO-10424</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -16658,7 +16682,7 @@
         <v>0</v>
       </c>
       <c r="K286" t="n">
-        <v>-36.95</v>
+        <v>-12.97</v>
       </c>
       <c r="L286" t="inlineStr">
         <is>
@@ -16679,7 +16703,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>PO-10425</t>
+          <t>PO-10426</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -16734,7 +16758,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>PO-10426</t>
+          <t>PO-10427</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -16789,7 +16813,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>PO-10427</t>
+          <t>PO-10428</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -16844,7 +16868,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>PO-10433</t>
+          <t>PO-10434</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -16899,7 +16923,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>PO-10434</t>
+          <t>PO-10435</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -16927,7 +16951,7 @@
         <v>0</v>
       </c>
       <c r="K291" t="n">
-        <v>257.98</v>
+        <v>281.96</v>
       </c>
       <c r="L291" t="inlineStr">
         <is>
@@ -16948,7 +16972,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>PO-10435</t>
+          <t>PO-10436</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -17003,7 +17027,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>PO-10436</t>
+          <t>PO-10437</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -17031,7 +17055,7 @@
         <v>0</v>
       </c>
       <c r="K293" t="n">
-        <v>-17.6</v>
+        <v>6.37</v>
       </c>
       <c r="L293" t="inlineStr">
         <is>
@@ -17052,7 +17076,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>PO-10438</t>
+          <t>PO-10439</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -17107,7 +17131,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>PO-10439</t>
+          <t>PO-10440</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -17162,7 +17186,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>PO-10442</t>
+          <t>PO-10443</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -17217,7 +17241,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>PO-10443</t>
+          <t>PO-10444</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -17272,7 +17296,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>PO-10445</t>
+          <t>PO-10446</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -17300,7 +17324,7 @@
         <v>0</v>
       </c>
       <c r="K298" t="n">
-        <v>976.34</v>
+        <v>1000.31</v>
       </c>
       <c r="L298" t="inlineStr">
         <is>
@@ -17321,7 +17345,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>PO-10446</t>
+          <t>PO-10447</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -17349,7 +17373,7 @@
         <v>0</v>
       </c>
       <c r="K299" t="n">
-        <v>4.28</v>
+        <v>28.26</v>
       </c>
       <c r="L299" t="inlineStr">
         <is>
@@ -17370,7 +17394,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>PO-10447</t>
+          <t>PO-10448</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -17425,7 +17449,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>PO-10448</t>
+          <t>PO-10449</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -17480,7 +17504,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>PO-10449</t>
+          <t>PO-10450</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -17535,12 +17559,12 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>PO-10450</t>
+          <t>PO-10451</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Em avaliação</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
@@ -17553,18 +17577,24 @@
           <t>2026-09-30T14:31:51.651151+00:00</t>
         </is>
       </c>
-      <c r="F303" t="inlineStr"/>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>2026-10-02T00:22:45.926736+00:00</t>
+        </is>
+      </c>
       <c r="G303" t="n">
         <v>49.98</v>
       </c>
-      <c r="H303" t="inlineStr"/>
-      <c r="I303" t="inlineStr"/>
+      <c r="H303" t="n">
+        <v>33.85</v>
+      </c>
+      <c r="I303" t="n">
+        <v>83.81999999999999</v>
+      </c>
       <c r="J303" t="b">
-        <v>0</v>
-      </c>
-      <c r="K303" t="n">
-        <v>70.56</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K303" t="inlineStr"/>
       <c r="L303" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -17584,7 +17614,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>PO-10454</t>
+          <t>PO-10455</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -17639,12 +17669,12 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>PO-10455</t>
+          <t>PO-10456</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Associado</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
@@ -17657,18 +17687,24 @@
           <t>2026-10-01T16:51:07.710434+00:00</t>
         </is>
       </c>
-      <c r="F305" t="inlineStr"/>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>2026-10-02T08:26:21.343284+00:00</t>
+        </is>
+      </c>
       <c r="G305" t="n">
         <v>51.24</v>
       </c>
-      <c r="H305" t="inlineStr"/>
-      <c r="I305" t="inlineStr"/>
+      <c r="H305" t="n">
+        <v>15.59</v>
+      </c>
+      <c r="I305" t="n">
+        <v>66.81999999999999</v>
+      </c>
       <c r="J305" t="b">
-        <v>0</v>
-      </c>
-      <c r="K305" t="n">
-        <v>45.49</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K305" t="inlineStr"/>
       <c r="L305" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -17688,7 +17724,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>PO-10456</t>
+          <t>PO-10457</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -17743,7 +17779,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>PO-10457</t>
+          <t>PO-10458</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -17798,7 +17834,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>PO-10458</t>
+          <t>PO-10459</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -17853,7 +17889,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>PO-10460</t>
+          <t>PO-10461</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -17881,7 +17917,7 @@
         <v>0</v>
       </c>
       <c r="K309" t="n">
-        <v>-66.68000000000001</v>
+        <v>-42.71</v>
       </c>
       <c r="L309" t="inlineStr">
         <is>
@@ -17902,7 +17938,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>PO-10461</t>
+          <t>PO-10462</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -17957,7 +17993,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>PO-10463</t>
+          <t>PO-10464</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -17985,7 +18021,7 @@
         <v>0</v>
       </c>
       <c r="K311" t="n">
-        <v>480.58</v>
+        <v>504.56</v>
       </c>
       <c r="L311" t="inlineStr">
         <is>
@@ -18006,7 +18042,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>PO-10467</t>
+          <t>PO-10468</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -18061,7 +18097,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>PO-10469</t>
+          <t>PO-10470</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -18089,7 +18125,7 @@
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>547.13</v>
+        <v>571.1</v>
       </c>
       <c r="L313" t="inlineStr">
         <is>
@@ -18110,7 +18146,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>PO-10470</t>
+          <t>PO-10471</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -18165,7 +18201,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>PO-10471</t>
+          <t>PO-10472</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -18220,7 +18256,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>PO-10472</t>
+          <t>PO-10473</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -18275,7 +18311,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>PO-10473</t>
+          <t>PO-10474</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -18330,7 +18366,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>PO-10474</t>
+          <t>PO-10475</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -18385,7 +18421,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>PO-10475</t>
+          <t>PO-10476</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -18440,7 +18476,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>PO-10476</t>
+          <t>PO-10477</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -18468,7 +18504,7 @@
         <v>0</v>
       </c>
       <c r="K320" t="n">
-        <v>905.84</v>
+        <v>929.8200000000001</v>
       </c>
       <c r="L320" t="inlineStr">
         <is>
@@ -18489,7 +18525,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>PO-10477</t>
+          <t>PO-10478</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -18517,7 +18553,7 @@
         <v>0</v>
       </c>
       <c r="K321" t="n">
-        <v>677.27</v>
+        <v>701.25</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -18538,7 +18574,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>PO-10478</t>
+          <t>PO-10479</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -18593,7 +18629,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>PO-10479</t>
+          <t>PO-10480</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -18648,7 +18684,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>PO-10480</t>
+          <t>PO-10481</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -18703,7 +18739,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>PO-10481</t>
+          <t>PO-10482</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -18731,7 +18767,7 @@
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>484.53</v>
+        <v>508.51</v>
       </c>
       <c r="L325" t="inlineStr">
         <is>
@@ -18752,7 +18788,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>PO-10484</t>
+          <t>PO-10485</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -18802,47 +18838,41 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>Delta Sports</t>
+          <t>Eterna Beleza</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>PO-10485</t>
+          <t>PO-10487</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Em avaliação</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>2026-08-19T09:53:22.177648+00:00</t>
+          <t>2026-08-19T00:55:46.780265+00:00</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>2026-08-20T05:51:53.283550+00:00</t>
-        </is>
-      </c>
-      <c r="F327" t="inlineStr">
-        <is>
-          <t>2026-08-23T20:43:07.922518+00:00</t>
-        </is>
-      </c>
+          <t>2026-08-21T02:30:47.843695+00:00</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr"/>
       <c r="G327" t="n">
-        <v>19.98</v>
-      </c>
-      <c r="H327" t="n">
-        <v>86.84999999999999</v>
-      </c>
-      <c r="I327" t="n">
-        <v>106.83</v>
-      </c>
+        <v>49.58</v>
+      </c>
+      <c r="H327" t="inlineStr"/>
+      <c r="I327" t="inlineStr"/>
       <c r="J327" t="b">
-        <v>1</v>
-      </c>
-      <c r="K327" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K327" t="n">
+        <v>1066.16</v>
+      </c>
       <c r="L327" t="inlineStr">
         <is>
           <t>2026-08</t>
@@ -18857,12 +18887,12 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>Eterna Beleza</t>
+          <t>Delta Sports</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>PO-10487</t>
+          <t>PO-10488</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -18872,27 +18902,27 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>2026-08-04T23:28:47.558849+00:00</t>
+          <t>2026-08-12T08:30:30.723409+00:00</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>2026-08-08T02:11:41.743500+00:00</t>
+          <t>2026-08-14T00:40:21.234609+00:00</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>2026-08-09T07:57:12.095994+00:00</t>
+          <t>2026-08-16T19:27:53.135754+00:00</t>
         </is>
       </c>
       <c r="G328" t="n">
-        <v>74.72</v>
+        <v>40.16</v>
       </c>
       <c r="H328" t="n">
-        <v>29.76</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I328" t="n">
-        <v>104.47</v>
+        <v>106.96</v>
       </c>
       <c r="J328" t="b">
         <v>1</v>
@@ -18905,7 +18935,7 @@
       </c>
       <c r="M328" t="inlineStr">
         <is>
-          <t>2026-S32</t>
+          <t>2026-S33</t>
         </is>
       </c>
     </row>
@@ -18917,42 +18947,36 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>PO-10488</t>
+          <t>PO-10489</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Associado</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>2026-09-02T20:07:43.581569+00:00</t>
+          <t>2026-09-23T12:19:38.213862+00:00</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>2026-09-04T00:25:37.978882+00:00</t>
-        </is>
-      </c>
-      <c r="F329" t="inlineStr">
-        <is>
-          <t>2026-09-05T20:45:36.532072+00:00</t>
-        </is>
-      </c>
+          <t>2026-09-26T01:53:00.738608+00:00</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr"/>
       <c r="G329" t="n">
-        <v>28.3</v>
-      </c>
-      <c r="H329" t="n">
-        <v>44.33</v>
-      </c>
-      <c r="I329" t="n">
-        <v>72.63</v>
-      </c>
+        <v>61.56</v>
+      </c>
+      <c r="H329" t="inlineStr"/>
+      <c r="I329" t="inlineStr"/>
       <c r="J329" t="b">
-        <v>1</v>
-      </c>
-      <c r="K329" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K329" t="n">
+        <v>214.76</v>
+      </c>
       <c r="L329" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -18960,19 +18984,19 @@
       </c>
       <c r="M329" t="inlineStr">
         <is>
-          <t>2026-S36</t>
+          <t>2026-S39</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>Fluxo Denim</t>
+          <t>Cedro Kids</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>PO-10489</t>
+          <t>PO-10490</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -18982,27 +19006,27 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>2026-09-29T00:11:14.881371+00:00</t>
+          <t>2026-08-19T17:15:07.605584+00:00</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>2026-09-29T13:18:28.144176+00:00</t>
+          <t>2026-08-21T19:28:39.829245+00:00</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>2026-09-29T21:47:37.635505+00:00</t>
+          <t>2026-08-26T04:38:30.998407+00:00</t>
         </is>
       </c>
       <c r="G330" t="n">
-        <v>13.12</v>
+        <v>50.23</v>
       </c>
       <c r="H330" t="n">
-        <v>8.49</v>
+        <v>105.16</v>
       </c>
       <c r="I330" t="n">
-        <v>21.61</v>
+        <v>155.39</v>
       </c>
       <c r="J330" t="b">
         <v>1</v>
@@ -19010,19 +19034,19 @@
       <c r="K330" t="inlineStr"/>
       <c r="L330" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="M330" t="inlineStr">
         <is>
-          <t>2026-S40</t>
+          <t>2026-S34</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>Bravo Casa</t>
+          <t>Alpha Moda</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -19032,52 +19056,46 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Em avaliação</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>2026-09-16T19:12:35.487348+00:00</t>
+          <t>2026-08-21T20:57:59.166000+00:00</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>2026-09-18T09:14:06.977187+00:00</t>
-        </is>
-      </c>
-      <c r="F331" t="inlineStr">
-        <is>
-          <t>2026-09-21T07:29:49.760764+00:00</t>
-        </is>
-      </c>
+          <t>2026-08-23T03:40:49.829977+00:00</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr"/>
       <c r="G331" t="n">
-        <v>38.03</v>
-      </c>
-      <c r="H331" t="n">
-        <v>70.26000000000001</v>
-      </c>
-      <c r="I331" t="n">
-        <v>108.29</v>
-      </c>
+        <v>30.71</v>
+      </c>
+      <c r="H331" t="inlineStr"/>
+      <c r="I331" t="inlineStr"/>
       <c r="J331" t="b">
-        <v>1</v>
-      </c>
-      <c r="K331" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K331" t="n">
+        <v>998.12</v>
+      </c>
       <c r="L331" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="M331" t="inlineStr">
         <is>
-          <t>2026-S38</t>
+          <t>2026-S34</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>Eterna Beleza</t>
+          <t>Fluxo Denim</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
@@ -19092,27 +19110,27 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>2026-09-04T10:41:45.474895+00:00</t>
+          <t>2026-08-12T22:59:08.192451+00:00</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>2026-09-07T10:22:02.081934+00:00</t>
+          <t>2026-08-13T09:15:07.499586+00:00</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>2026-09-07T22:27:42.436228+00:00</t>
+          <t>2026-08-17T18:14:17.186973+00:00</t>
         </is>
       </c>
       <c r="G332" t="n">
-        <v>71.67</v>
+        <v>10.27</v>
       </c>
       <c r="H332" t="n">
-        <v>12.09</v>
+        <v>104.99</v>
       </c>
       <c r="I332" t="n">
-        <v>83.77</v>
+        <v>115.25</v>
       </c>
       <c r="J332" t="b">
         <v>1</v>
@@ -19120,12 +19138,12 @@
       <c r="K332" t="inlineStr"/>
       <c r="L332" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="M332" t="inlineStr">
         <is>
-          <t>2026-S36</t>
+          <t>2026-S33</t>
         </is>
       </c>
     </row>
@@ -19330,7 +19348,7 @@
         <v>0</v>
       </c>
       <c r="K336" t="n">
-        <v>206.87</v>
+        <v>230.84</v>
       </c>
       <c r="L336" t="inlineStr">
         <is>
@@ -19379,7 +19397,7 @@
         <v>0</v>
       </c>
       <c r="K337" t="n">
-        <v>797.5</v>
+        <v>821.47</v>
       </c>
       <c r="L337" t="inlineStr">
         <is>
@@ -19758,7 +19776,7 @@
         <v>0</v>
       </c>
       <c r="K344" t="n">
-        <v>1015.1</v>
+        <v>1039.08</v>
       </c>
       <c r="L344" t="inlineStr">
         <is>
@@ -19917,7 +19935,7 @@
         <v>0</v>
       </c>
       <c r="K347" t="n">
-        <v>488.68</v>
+        <v>512.66</v>
       </c>
       <c r="L347" t="inlineStr">
         <is>
@@ -19966,7 +19984,7 @@
         <v>0</v>
       </c>
       <c r="K348" t="n">
-        <v>52.62</v>
+        <v>76.59</v>
       </c>
       <c r="L348" t="inlineStr">
         <is>
@@ -20015,7 +20033,7 @@
         <v>0</v>
       </c>
       <c r="K349" t="n">
-        <v>399.22</v>
+        <v>423.2</v>
       </c>
       <c r="L349" t="inlineStr">
         <is>
@@ -20284,7 +20302,7 @@
         <v>0</v>
       </c>
       <c r="K354" t="n">
-        <v>131.76</v>
+        <v>155.74</v>
       </c>
       <c r="L354" t="inlineStr">
         <is>
@@ -20498,7 +20516,7 @@
         <v>0</v>
       </c>
       <c r="K358" t="n">
-        <v>1236.66</v>
+        <v>1260.63</v>
       </c>
       <c r="L358" t="inlineStr">
         <is>
@@ -20547,7 +20565,7 @@
         <v>0</v>
       </c>
       <c r="K359" t="n">
-        <v>502.54</v>
+        <v>526.51</v>
       </c>
       <c r="L359" t="inlineStr">
         <is>
@@ -20816,7 +20834,7 @@
         <v>0</v>
       </c>
       <c r="K364" t="n">
-        <v>8.800000000000001</v>
+        <v>32.78</v>
       </c>
       <c r="L364" t="inlineStr">
         <is>
@@ -20975,7 +20993,7 @@
         <v>0</v>
       </c>
       <c r="K367" t="n">
-        <v>102.5</v>
+        <v>126.47</v>
       </c>
       <c r="L367" t="inlineStr">
         <is>
@@ -21024,7 +21042,7 @@
         <v>0</v>
       </c>
       <c r="K368" t="n">
-        <v>-38.89</v>
+        <v>-14.92</v>
       </c>
       <c r="L368" t="inlineStr">
         <is>
@@ -21073,7 +21091,7 @@
         <v>0</v>
       </c>
       <c r="K369" t="n">
-        <v>1074.93</v>
+        <v>1098.91</v>
       </c>
       <c r="L369" t="inlineStr">
         <is>
@@ -21232,7 +21250,7 @@
         <v>0</v>
       </c>
       <c r="K372" t="n">
-        <v>-17.13</v>
+        <v>6.85</v>
       </c>
       <c r="L372" t="inlineStr">
         <is>
@@ -21831,7 +21849,7 @@
         <v>0</v>
       </c>
       <c r="K383" t="n">
-        <v>69.93000000000001</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="L383" t="inlineStr">
         <is>
@@ -21990,7 +22008,7 @@
         <v>0</v>
       </c>
       <c r="K386" t="n">
-        <v>124.91</v>
+        <v>148.89</v>
       </c>
       <c r="L386" t="inlineStr">
         <is>
@@ -22181,7 +22199,7 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D390" t="inlineStr">
@@ -22194,18 +22212,24 @@
           <t>2026-09-28T23:50:07.769529+00:00</t>
         </is>
       </c>
-      <c r="F390" t="inlineStr"/>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>2026-10-02T10:36:19.794849+00:00</t>
+        </is>
+      </c>
       <c r="G390" t="n">
         <v>14.25</v>
       </c>
-      <c r="H390" t="inlineStr"/>
-      <c r="I390" t="inlineStr"/>
+      <c r="H390" t="n">
+        <v>82.77</v>
+      </c>
+      <c r="I390" t="n">
+        <v>97.02</v>
+      </c>
       <c r="J390" t="b">
-        <v>0</v>
-      </c>
-      <c r="K390" t="n">
-        <v>73.53</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K390" t="inlineStr"/>
       <c r="L390" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -22308,7 +22332,7 @@
         <v>0</v>
       </c>
       <c r="K392" t="n">
-        <v>1080.81</v>
+        <v>1104.79</v>
       </c>
       <c r="L392" t="inlineStr">
         <is>
@@ -22334,7 +22358,7 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
@@ -22347,18 +22371,24 @@
           <t>2026-09-27T19:31:16.868570+00:00</t>
         </is>
       </c>
-      <c r="F393" t="inlineStr"/>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>2026-10-02T06:40:44.266323+00:00</t>
+        </is>
+      </c>
       <c r="G393" t="n">
         <v>23.06</v>
       </c>
-      <c r="H393" t="inlineStr"/>
-      <c r="I393" t="inlineStr"/>
+      <c r="H393" t="n">
+        <v>107.16</v>
+      </c>
+      <c r="I393" t="n">
+        <v>130.22</v>
+      </c>
       <c r="J393" t="b">
-        <v>0</v>
-      </c>
-      <c r="K393" t="n">
-        <v>110.65</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K393" t="inlineStr"/>
       <c r="L393" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -22461,7 +22491,7 @@
         <v>0</v>
       </c>
       <c r="K395" t="n">
-        <v>-52.62</v>
+        <v>-28.64</v>
       </c>
       <c r="L395" t="inlineStr">
         <is>
@@ -22675,7 +22705,7 @@
         <v>0</v>
       </c>
       <c r="K399" t="n">
-        <v>104.63</v>
+        <v>128.61</v>
       </c>
       <c r="L399" t="inlineStr">
         <is>
@@ -22724,7 +22754,7 @@
         <v>0</v>
       </c>
       <c r="K400" t="n">
-        <v>-88.23</v>
+        <v>-64.25</v>
       </c>
       <c r="L400" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualiza painel (2026-10-15 11:18 UTC)
</commit_message>
<xml_diff>
--- a/dados/status_atual.xlsx
+++ b/dados/status_atual.xlsx
@@ -452,7 +452,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>95.40000000000001</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -463,7 +463,7 @@
         <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3">
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>82.5</v>
+        <v>82.3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -484,7 +484,7 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>303</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>73</v>
+        <v>72.8</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -505,7 +505,7 @@
         <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>312</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>61.1</v>
+        <v>60.4</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -526,7 +526,7 @@
         <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>261</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>44.6</v>
+        <v>44.8</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>26.6</v>
+        <v>25.2</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -568,7 +568,7 @@
         <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -644,10 +644,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E2" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F2" t="n">
         <v>2</v>
@@ -656,7 +656,7 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>95.90000000000001</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3">
@@ -676,10 +676,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E3" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F3" t="n">
         <v>2</v>
@@ -688,7 +688,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>97.2</v>
+        <v>97.3</v>
       </c>
     </row>
     <row r="4">
@@ -708,10 +708,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E4" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F4" t="n">
         <v>5</v>
@@ -720,7 +720,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>93.8</v>
+        <v>93.90000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -740,19 +740,19 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E5" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>94.59999999999999</v>
+        <v>96.5</v>
       </c>
     </row>
     <row r="6">
@@ -772,10 +772,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E6" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F6" t="n">
         <v>10</v>
@@ -784,7 +784,7 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>83.3</v>
+        <v>82.8</v>
       </c>
     </row>
     <row r="7">
@@ -804,10 +804,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E7" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F7" t="n">
         <v>12</v>
@@ -816,7 +816,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>85.2</v>
+        <v>84.8</v>
       </c>
     </row>
     <row r="8">
@@ -836,19 +836,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E8" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F8" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>76.90000000000001</v>
+        <v>77.5</v>
       </c>
     </row>
     <row r="9">
@@ -868,10 +868,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E9" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F9" t="n">
         <v>11</v>
@@ -880,7 +880,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>84.5</v>
+        <v>84.09999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -900,10 +900,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E10" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F10" t="n">
         <v>19</v>
@@ -912,7 +912,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>62.7</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11">
@@ -932,19 +932,19 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E11" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F11" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>52.9</v>
+        <v>50.7</v>
       </c>
     </row>
     <row r="12">
@@ -964,19 +964,19 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E12" t="n">
         <v>51</v>
       </c>
       <c r="F12" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>63.7</v>
+        <v>64.59999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -996,10 +996,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E13" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F13" t="n">
         <v>21</v>
@@ -1008,7 +1008,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>65</v>
+        <v>64.40000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -1031,16 +1031,16 @@
         <v>69</v>
       </c>
       <c r="E14" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F14" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>36.2</v>
+        <v>37.7</v>
       </c>
     </row>
     <row r="15">
@@ -1095,16 +1095,16 @@
         <v>105</v>
       </c>
       <c r="E16" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F16" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>47.6</v>
+        <v>46.7</v>
       </c>
     </row>
     <row r="17">
@@ -1156,10 +1156,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E18" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F18" t="n">
         <v>35</v>
@@ -1168,7 +1168,7 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>27.1</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="19">
@@ -1191,16 +1191,16 @@
         <v>67</v>
       </c>
       <c r="E19" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F19" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>28.4</v>
+        <v>26.9</v>
       </c>
     </row>
     <row r="20">
@@ -1223,16 +1223,16 @@
         <v>77</v>
       </c>
       <c r="E20" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F20" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>29.9</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="21">
@@ -1284,10 +1284,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E22" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F22" t="n">
         <v>20</v>
@@ -1296,7 +1296,7 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>70.09999999999999</v>
+        <v>70.59999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -1316,19 +1316,19 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E23" t="n">
         <v>60</v>
       </c>
       <c r="F23" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>73.2</v>
+        <v>72.3</v>
       </c>
     </row>
     <row r="24">
@@ -1348,19 +1348,19 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E24" t="n">
         <v>72</v>
       </c>
       <c r="F24" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>83.7</v>
+        <v>82.8</v>
       </c>
     </row>
     <row r="25">
@@ -1380,10 +1380,10 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E25" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F25" t="n">
         <v>27</v>
@@ -1392,7 +1392,7 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>64.90000000000001</v>
+        <v>65.40000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1406,7 +1406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M397"/>
+  <dimension ref="A1:M396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1622,7 +1622,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>983.64</v>
+        <v>1007.62</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -1781,7 +1781,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>1094.76</v>
+        <v>1118.75</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -1830,7 +1830,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>218.97</v>
+        <v>242.96</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>21.71</v>
+        <v>45.69</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -1928,7 +1928,7 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>1473.64</v>
+        <v>1497.63</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>294.14</v>
+        <v>318.13</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -2008,12 +2008,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-10T17:07:19.707982+00:00</t>
+          <t>2026-10-17T21:33:54.969945+00:00</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-10-12T16:22:49.581282+00:00</t>
+          <t>2026-10-19T20:49:24.843245+00:00</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -2026,7 +2026,7 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>90.2</v>
+        <v>-58.26</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-S41</t>
+          <t>2026-S42</t>
         </is>
       </c>
     </row>
@@ -2075,7 +2075,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>880.1</v>
+        <v>904.09</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -2124,7 +2124,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>1237.14</v>
+        <v>1261.12</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -2503,7 +2503,7 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>93.98999999999999</v>
+        <v>117.98</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -2717,7 +2717,7 @@
         <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>330.04</v>
+        <v>354.03</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -2986,7 +2986,7 @@
         <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>1677.41</v>
+        <v>1701.4</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -3420,7 +3420,7 @@
         <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>-31.92</v>
+        <v>-7.93</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -3524,7 +3524,7 @@
         <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>-3.84</v>
+        <v>20.14</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>417.62</v>
+        <v>441.61</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -3787,7 +3787,7 @@
         <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>601.98</v>
+        <v>625.97</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
@@ -4111,7 +4111,7 @@
         <v>0</v>
       </c>
       <c r="K51" t="n">
-        <v>1050.61</v>
+        <v>1074.6</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -4215,7 +4215,7 @@
         <v>0</v>
       </c>
       <c r="K53" t="n">
-        <v>1084.93</v>
+        <v>1108.92</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -4319,7 +4319,7 @@
         <v>0</v>
       </c>
       <c r="K55" t="n">
-        <v>-46.46</v>
+        <v>-22.48</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
         <v>0</v>
       </c>
       <c r="K57" t="n">
-        <v>-82.86</v>
+        <v>-58.87</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
@@ -4472,7 +4472,7 @@
         <v>0</v>
       </c>
       <c r="K58" t="n">
-        <v>1655.57</v>
+        <v>1679.55</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
@@ -4686,7 +4686,7 @@
         <v>0</v>
       </c>
       <c r="K62" t="n">
-        <v>763.04</v>
+        <v>787.03</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -4845,7 +4845,7 @@
         <v>0</v>
       </c>
       <c r="K65" t="n">
-        <v>-16.37</v>
+        <v>7.62</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
@@ -4894,7 +4894,7 @@
         <v>0</v>
       </c>
       <c r="K66" t="n">
-        <v>883.02</v>
+        <v>907.01</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
@@ -4943,7 +4943,7 @@
         <v>0</v>
       </c>
       <c r="K67" t="n">
-        <v>158.8</v>
+        <v>182.79</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
@@ -5047,7 +5047,7 @@
         <v>0</v>
       </c>
       <c r="K69" t="n">
-        <v>31.79</v>
+        <v>55.77</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -5371,7 +5371,7 @@
         <v>0</v>
       </c>
       <c r="K75" t="n">
-        <v>47.62</v>
+        <v>71.61</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -5695,7 +5695,7 @@
         <v>0</v>
       </c>
       <c r="K81" t="n">
-        <v>1502.92</v>
+        <v>1526.91</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
@@ -5964,7 +5964,7 @@
         <v>0</v>
       </c>
       <c r="K86" t="n">
-        <v>14.24</v>
+        <v>38.23</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -5980,7 +5980,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Eterna Beleza</t>
+          <t>Cedro Kids</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -6000,22 +6000,22 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>2026-10-01T12:09:19.876475+00:00</t>
+          <t>2026-10-01T03:43:15.853702+00:00</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2026-10-02T12:18:20.190696+00:00</t>
+          <t>2026-10-01T21:37:23.769557+00:00</t>
         </is>
       </c>
       <c r="G87" t="n">
-        <v>32.6</v>
+        <v>24.17</v>
       </c>
       <c r="H87" t="n">
-        <v>24.15</v>
+        <v>17.9</v>
       </c>
       <c r="I87" t="n">
-        <v>56.75</v>
+        <v>42.07</v>
       </c>
       <c r="J87" t="b">
         <v>1</v>
@@ -6288,7 +6288,7 @@
         <v>0</v>
       </c>
       <c r="K92" t="n">
-        <v>-65.23</v>
+        <v>-41.24</v>
       </c>
       <c r="L92" t="inlineStr">
         <is>
@@ -6337,7 +6337,7 @@
         <v>0</v>
       </c>
       <c r="K93" t="n">
-        <v>1444.89</v>
+        <v>1468.88</v>
       </c>
       <c r="L93" t="inlineStr">
         <is>
@@ -6386,7 +6386,7 @@
         <v>0</v>
       </c>
       <c r="K94" t="n">
-        <v>1096.3</v>
+        <v>1120.29</v>
       </c>
       <c r="L94" t="inlineStr">
         <is>
@@ -6600,7 +6600,7 @@
         <v>0</v>
       </c>
       <c r="K98" t="n">
-        <v>191.71</v>
+        <v>215.7</v>
       </c>
       <c r="L98" t="inlineStr">
         <is>
@@ -7034,7 +7034,7 @@
         <v>0</v>
       </c>
       <c r="K106" t="n">
-        <v>763.1</v>
+        <v>787.09</v>
       </c>
       <c r="L106" t="inlineStr">
         <is>
@@ -7248,7 +7248,7 @@
         <v>0</v>
       </c>
       <c r="K110" t="n">
-        <v>248.17</v>
+        <v>272.16</v>
       </c>
       <c r="L110" t="inlineStr">
         <is>
@@ -7682,7 +7682,7 @@
         <v>0</v>
       </c>
       <c r="K118" t="n">
-        <v>30.9</v>
+        <v>54.89</v>
       </c>
       <c r="L118" t="inlineStr">
         <is>
@@ -7873,7 +7873,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Associado</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -7886,18 +7886,24 @@
           <t>2026-10-12T13:09:15.202202+00:00</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>2026-10-15T10:50:37.894047+00:00</t>
+        </is>
+      </c>
       <c r="G122" t="n">
         <v>42.76</v>
       </c>
-      <c r="H122" t="inlineStr"/>
-      <c r="I122" t="inlineStr"/>
+      <c r="H122" t="n">
+        <v>69.69</v>
+      </c>
+      <c r="I122" t="n">
+        <v>112.45</v>
+      </c>
       <c r="J122" t="b">
-        <v>0</v>
-      </c>
-      <c r="K122" t="n">
-        <v>88.92</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
           <t>2026-10</t>
@@ -8000,7 +8006,7 @@
         <v>0</v>
       </c>
       <c r="K124" t="n">
-        <v>1073.03</v>
+        <v>1097.02</v>
       </c>
       <c r="L124" t="inlineStr">
         <is>
@@ -8136,7 +8142,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Em avaliação</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -8149,18 +8155,24 @@
           <t>2026-10-13T18:53:04.059609+00:00</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr"/>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>2026-10-14T20:13:34.548338+00:00</t>
+        </is>
+      </c>
       <c r="G127" t="n">
         <v>6.89</v>
       </c>
-      <c r="H127" t="inlineStr"/>
-      <c r="I127" t="inlineStr"/>
+      <c r="H127" t="n">
+        <v>25.34</v>
+      </c>
+      <c r="I127" t="n">
+        <v>32.23</v>
+      </c>
       <c r="J127" t="b">
-        <v>0</v>
-      </c>
-      <c r="K127" t="n">
-        <v>23.32</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr">
         <is>
           <t>2026-10</t>
@@ -8318,7 +8330,7 @@
         <v>0</v>
       </c>
       <c r="K130" t="n">
-        <v>1494.61</v>
+        <v>1518.59</v>
       </c>
       <c r="L130" t="inlineStr">
         <is>
@@ -8367,7 +8379,7 @@
         <v>0</v>
       </c>
       <c r="K131" t="n">
-        <v>312.8</v>
+        <v>336.79</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
@@ -8416,7 +8428,7 @@
         <v>0</v>
       </c>
       <c r="K132" t="n">
-        <v>-101.67</v>
+        <v>-77.68000000000001</v>
       </c>
       <c r="L132" t="inlineStr">
         <is>
@@ -8685,7 +8697,7 @@
         <v>0</v>
       </c>
       <c r="K137" t="n">
-        <v>1175.13</v>
+        <v>1199.12</v>
       </c>
       <c r="L137" t="inlineStr">
         <is>
@@ -8734,7 +8746,7 @@
         <v>0</v>
       </c>
       <c r="K138" t="n">
-        <v>1668.57</v>
+        <v>1692.56</v>
       </c>
       <c r="L138" t="inlineStr">
         <is>
@@ -8815,7 +8827,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Em avaliação</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -8828,18 +8840,24 @@
           <t>2026-10-13T02:09:19.393552+00:00</t>
         </is>
       </c>
-      <c r="F140" t="inlineStr"/>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>2026-10-15T03:13:51.990655+00:00</t>
+        </is>
+      </c>
       <c r="G140" t="n">
         <v>55.84</v>
       </c>
-      <c r="H140" t="inlineStr"/>
-      <c r="I140" t="inlineStr"/>
+      <c r="H140" t="n">
+        <v>49.08</v>
+      </c>
+      <c r="I140" t="n">
+        <v>104.92</v>
+      </c>
       <c r="J140" t="b">
-        <v>0</v>
-      </c>
-      <c r="K140" t="n">
-        <v>89.01000000000001</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr">
         <is>
           <t>2026-10</t>
@@ -9107,7 +9125,7 @@
         <v>0</v>
       </c>
       <c r="K145" t="n">
-        <v>274.2</v>
+        <v>298.19</v>
       </c>
       <c r="L145" t="inlineStr">
         <is>
@@ -9321,7 +9339,7 @@
         <v>0</v>
       </c>
       <c r="K149" t="n">
-        <v>1.73</v>
+        <v>25.72</v>
       </c>
       <c r="L149" t="inlineStr">
         <is>
@@ -9755,7 +9773,7 @@
         <v>0</v>
       </c>
       <c r="K157" t="n">
-        <v>593.95</v>
+        <v>617.9400000000001</v>
       </c>
       <c r="L157" t="inlineStr">
         <is>
@@ -9859,7 +9877,7 @@
         <v>0</v>
       </c>
       <c r="K159" t="n">
-        <v>381.88</v>
+        <v>405.86</v>
       </c>
       <c r="L159" t="inlineStr">
         <is>
@@ -9963,7 +9981,7 @@
         <v>0</v>
       </c>
       <c r="K161" t="n">
-        <v>1261.61</v>
+        <v>1285.59</v>
       </c>
       <c r="L161" t="inlineStr">
         <is>
@@ -10067,7 +10085,7 @@
         <v>0</v>
       </c>
       <c r="K163" t="n">
-        <v>567.51</v>
+        <v>591.49</v>
       </c>
       <c r="L163" t="inlineStr">
         <is>
@@ -10171,7 +10189,7 @@
         <v>0</v>
       </c>
       <c r="K165" t="n">
-        <v>-32.96</v>
+        <v>-8.98</v>
       </c>
       <c r="L165" t="inlineStr">
         <is>
@@ -10275,7 +10293,7 @@
         <v>0</v>
       </c>
       <c r="K167" t="n">
-        <v>1232.09</v>
+        <v>1256.08</v>
       </c>
       <c r="L167" t="inlineStr">
         <is>
@@ -10654,7 +10672,7 @@
         <v>0</v>
       </c>
       <c r="K174" t="n">
-        <v>1168.2</v>
+        <v>1192.19</v>
       </c>
       <c r="L174" t="inlineStr">
         <is>
@@ -11198,7 +11216,7 @@
         <v>0</v>
       </c>
       <c r="K184" t="n">
-        <v>994.89</v>
+        <v>1018.87</v>
       </c>
       <c r="L184" t="inlineStr">
         <is>
@@ -11302,7 +11320,7 @@
         <v>0</v>
       </c>
       <c r="K186" t="n">
-        <v>-14.35</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="L186" t="inlineStr">
         <is>
@@ -11406,7 +11424,7 @@
         <v>0</v>
       </c>
       <c r="K188" t="n">
-        <v>125.05</v>
+        <v>149.04</v>
       </c>
       <c r="L188" t="inlineStr">
         <is>
@@ -11565,7 +11583,7 @@
         <v>0</v>
       </c>
       <c r="K191" t="n">
-        <v>71.27</v>
+        <v>95.26000000000001</v>
       </c>
       <c r="L191" t="inlineStr">
         <is>
@@ -11614,7 +11632,7 @@
         <v>0</v>
       </c>
       <c r="K192" t="n">
-        <v>-99.83</v>
+        <v>-75.84999999999999</v>
       </c>
       <c r="L192" t="inlineStr">
         <is>
@@ -11718,7 +11736,7 @@
         <v>0</v>
       </c>
       <c r="K194" t="n">
-        <v>44.91</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="L194" t="inlineStr">
         <is>
@@ -11822,7 +11840,7 @@
         <v>0</v>
       </c>
       <c r="K196" t="n">
-        <v>1423.07</v>
+        <v>1447.06</v>
       </c>
       <c r="L196" t="inlineStr">
         <is>
@@ -12036,7 +12054,7 @@
         <v>0</v>
       </c>
       <c r="K200" t="n">
-        <v>1742.12</v>
+        <v>1766.11</v>
       </c>
       <c r="L200" t="inlineStr">
         <is>
@@ -12085,7 +12103,7 @@
         <v>0</v>
       </c>
       <c r="K201" t="n">
-        <v>-46.44</v>
+        <v>-22.46</v>
       </c>
       <c r="L201" t="inlineStr">
         <is>
@@ -12134,7 +12152,7 @@
         <v>0</v>
       </c>
       <c r="K202" t="n">
-        <v>235.33</v>
+        <v>259.31</v>
       </c>
       <c r="L202" t="inlineStr">
         <is>
@@ -12458,7 +12476,7 @@
         <v>0</v>
       </c>
       <c r="K208" t="n">
-        <v>265.67</v>
+        <v>289.66</v>
       </c>
       <c r="L208" t="inlineStr">
         <is>
@@ -12507,7 +12525,7 @@
         <v>0</v>
       </c>
       <c r="K209" t="n">
-        <v>-18.71</v>
+        <v>5.28</v>
       </c>
       <c r="L209" t="inlineStr">
         <is>
@@ -12556,7 +12574,7 @@
         <v>0</v>
       </c>
       <c r="K210" t="n">
-        <v>45.93</v>
+        <v>69.92</v>
       </c>
       <c r="L210" t="inlineStr">
         <is>
@@ -12660,7 +12678,7 @@
         <v>0</v>
       </c>
       <c r="K212" t="n">
-        <v>1335.43</v>
+        <v>1359.41</v>
       </c>
       <c r="L212" t="inlineStr">
         <is>
@@ -12764,7 +12782,7 @@
         <v>0</v>
       </c>
       <c r="K214" t="n">
-        <v>4.98</v>
+        <v>28.96</v>
       </c>
       <c r="L214" t="inlineStr">
         <is>
@@ -12813,7 +12831,7 @@
         <v>0</v>
       </c>
       <c r="K215" t="n">
-        <v>1064.78</v>
+        <v>1088.77</v>
       </c>
       <c r="L215" t="inlineStr">
         <is>
@@ -13027,7 +13045,7 @@
         <v>0</v>
       </c>
       <c r="K219" t="n">
-        <v>-34.8</v>
+        <v>-10.81</v>
       </c>
       <c r="L219" t="inlineStr">
         <is>
@@ -13296,7 +13314,7 @@
         <v>0</v>
       </c>
       <c r="K224" t="n">
-        <v>1454.54</v>
+        <v>1478.53</v>
       </c>
       <c r="L224" t="inlineStr">
         <is>
@@ -13400,7 +13418,7 @@
         <v>0</v>
       </c>
       <c r="K226" t="n">
-        <v>-49.88</v>
+        <v>-25.9</v>
       </c>
       <c r="L226" t="inlineStr">
         <is>
@@ -13504,7 +13522,7 @@
         <v>0</v>
       </c>
       <c r="K228" t="n">
-        <v>1575.1</v>
+        <v>1599.08</v>
       </c>
       <c r="L228" t="inlineStr">
         <is>
@@ -13553,7 +13571,7 @@
         <v>0</v>
       </c>
       <c r="K229" t="n">
-        <v>899.46</v>
+        <v>923.45</v>
       </c>
       <c r="L229" t="inlineStr">
         <is>
@@ -13712,7 +13730,7 @@
         <v>0</v>
       </c>
       <c r="K232" t="n">
-        <v>1572</v>
+        <v>1595.99</v>
       </c>
       <c r="L232" t="inlineStr">
         <is>
@@ -13981,7 +13999,7 @@
         <v>0</v>
       </c>
       <c r="K237" t="n">
-        <v>508.35</v>
+        <v>532.34</v>
       </c>
       <c r="L237" t="inlineStr">
         <is>
@@ -14030,7 +14048,7 @@
         <v>0</v>
       </c>
       <c r="K238" t="n">
-        <v>1620.25</v>
+        <v>1644.24</v>
       </c>
       <c r="L238" t="inlineStr">
         <is>
@@ -14079,7 +14097,7 @@
         <v>0</v>
       </c>
       <c r="K239" t="n">
-        <v>178.78</v>
+        <v>202.77</v>
       </c>
       <c r="L239" t="inlineStr">
         <is>
@@ -14238,7 +14256,7 @@
         <v>0</v>
       </c>
       <c r="K242" t="n">
-        <v>-63.08</v>
+        <v>-39.1</v>
       </c>
       <c r="L242" t="inlineStr">
         <is>
@@ -14562,7 +14580,7 @@
         <v>0</v>
       </c>
       <c r="K248" t="n">
-        <v>27.27</v>
+        <v>51.26</v>
       </c>
       <c r="L248" t="inlineStr">
         <is>
@@ -14808,37 +14826,31 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Em avaliação</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>2026-10-04T10:17:28.209232+00:00</t>
+          <t>2026-10-18T13:23:39.846226+00:00</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>2026-10-07T16:04:50.016311+00:00</t>
-        </is>
-      </c>
-      <c r="F253" t="inlineStr">
-        <is>
-          <t>2026-10-08T07:08:56.289812+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-20T08:55:43.732851+00:00</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr"/>
       <c r="G253" t="n">
-        <v>77.79000000000001</v>
-      </c>
-      <c r="H253" t="n">
-        <v>15.07</v>
-      </c>
-      <c r="I253" t="n">
-        <v>92.86</v>
-      </c>
+        <v>43.53</v>
+      </c>
+      <c r="H253" t="inlineStr"/>
+      <c r="I253" t="inlineStr"/>
       <c r="J253" t="b">
-        <v>1</v>
-      </c>
-      <c r="K253" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K253" t="n">
+        <v>-74.09</v>
+      </c>
       <c r="L253" t="inlineStr">
         <is>
           <t>2026-10</t>
@@ -14846,7 +14858,7 @@
       </c>
       <c r="M253" t="inlineStr">
         <is>
-          <t>2026-S40</t>
+          <t>2026-S42</t>
         </is>
       </c>
     </row>
@@ -14868,27 +14880,27 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>2026-08-18T16:09:14.191751+00:00</t>
+          <t>2026-09-15T06:53:05.711425+00:00</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>2026-08-19T00:47:47.640722+00:00</t>
+          <t>2026-09-16T17:28:04.173575+00:00</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>2026-08-20T13:03:23.330378+00:00</t>
+          <t>2026-09-17T16:26:34.154727+00:00</t>
         </is>
       </c>
       <c r="G254" t="n">
-        <v>8.640000000000001</v>
+        <v>34.58</v>
       </c>
       <c r="H254" t="n">
-        <v>36.26</v>
+        <v>22.97</v>
       </c>
       <c r="I254" t="n">
-        <v>44.9</v>
+        <v>57.56</v>
       </c>
       <c r="J254" t="b">
         <v>1</v>
@@ -14896,12 +14908,12 @@
       <c r="K254" t="inlineStr"/>
       <c r="L254" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="M254" t="inlineStr">
         <is>
-          <t>2026-S34</t>
+          <t>2026-S38</t>
         </is>
       </c>
     </row>
@@ -15216,7 +15228,7 @@
         <v>0</v>
       </c>
       <c r="K260" t="n">
-        <v>64.84999999999999</v>
+        <v>88.84</v>
       </c>
       <c r="L260" t="inlineStr">
         <is>
@@ -15265,7 +15277,7 @@
         <v>0</v>
       </c>
       <c r="K261" t="n">
-        <v>84.94</v>
+        <v>108.92</v>
       </c>
       <c r="L261" t="inlineStr">
         <is>
@@ -15534,7 +15546,7 @@
         <v>0</v>
       </c>
       <c r="K266" t="n">
-        <v>1030.94</v>
+        <v>1054.93</v>
       </c>
       <c r="L266" t="inlineStr">
         <is>
@@ -15638,7 +15650,7 @@
         <v>0</v>
       </c>
       <c r="K268" t="n">
-        <v>1699.63</v>
+        <v>1723.62</v>
       </c>
       <c r="L268" t="inlineStr">
         <is>
@@ -15742,7 +15754,7 @@
         <v>0</v>
       </c>
       <c r="K270" t="n">
-        <v>1199.55</v>
+        <v>1223.54</v>
       </c>
       <c r="L270" t="inlineStr">
         <is>
@@ -15791,7 +15803,7 @@
         <v>0</v>
       </c>
       <c r="K271" t="n">
-        <v>1670.8</v>
+        <v>1694.79</v>
       </c>
       <c r="L271" t="inlineStr">
         <is>
@@ -15840,7 +15852,7 @@
         <v>0</v>
       </c>
       <c r="K272" t="n">
-        <v>300.1</v>
+        <v>324.08</v>
       </c>
       <c r="L272" t="inlineStr">
         <is>
@@ -15889,7 +15901,7 @@
         <v>0</v>
       </c>
       <c r="K273" t="n">
-        <v>1416.5</v>
+        <v>1440.49</v>
       </c>
       <c r="L273" t="inlineStr">
         <is>
@@ -15993,7 +16005,7 @@
         <v>0</v>
       </c>
       <c r="K275" t="n">
-        <v>746.36</v>
+        <v>770.34</v>
       </c>
       <c r="L275" t="inlineStr">
         <is>
@@ -16042,7 +16054,7 @@
         <v>0</v>
       </c>
       <c r="K276" t="n">
-        <v>116.93</v>
+        <v>140.92</v>
       </c>
       <c r="L276" t="inlineStr">
         <is>
@@ -16366,7 +16378,7 @@
         <v>0</v>
       </c>
       <c r="K282" t="n">
-        <v>1205.33</v>
+        <v>1229.31</v>
       </c>
       <c r="L282" t="inlineStr">
         <is>
@@ -16722,7 +16734,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Associado</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -16735,18 +16747,24 @@
           <t>2026-10-10T13:59:28.879122+00:00</t>
         </is>
       </c>
-      <c r="F289" t="inlineStr"/>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>2026-10-14T20:19:41.163147+00:00</t>
+        </is>
+      </c>
       <c r="G289" t="n">
         <v>45.04</v>
       </c>
-      <c r="H289" t="inlineStr"/>
-      <c r="I289" t="inlineStr"/>
+      <c r="H289" t="n">
+        <v>102.34</v>
+      </c>
+      <c r="I289" t="n">
+        <v>147.38</v>
+      </c>
       <c r="J289" t="b">
-        <v>0</v>
-      </c>
-      <c r="K289" t="n">
-        <v>138.37</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K289" t="inlineStr"/>
       <c r="L289" t="inlineStr">
         <is>
           <t>2026-10</t>
@@ -16849,7 +16867,7 @@
         <v>0</v>
       </c>
       <c r="K291" t="n">
-        <v>12.2</v>
+        <v>36.18</v>
       </c>
       <c r="L291" t="inlineStr">
         <is>
@@ -16898,7 +16916,7 @@
         <v>0</v>
       </c>
       <c r="K292" t="n">
-        <v>880.55</v>
+        <v>904.53</v>
       </c>
       <c r="L292" t="inlineStr">
         <is>
@@ -17034,52 +17052,46 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Associado</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>2026-08-28T02:08:47.489081+00:00</t>
+          <t>2026-10-17T06:26:24.489716+00:00</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>2026-08-31T13:57:00.431691+00:00</t>
-        </is>
-      </c>
-      <c r="F295" t="inlineStr">
-        <is>
-          <t>2026-09-01T21:54:10.546246+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-19T20:04:27.778683+00:00</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr"/>
       <c r="G295" t="n">
-        <v>83.8</v>
-      </c>
-      <c r="H295" t="n">
-        <v>31.95</v>
-      </c>
-      <c r="I295" t="n">
-        <v>115.76</v>
-      </c>
+        <v>61.63</v>
+      </c>
+      <c r="H295" t="inlineStr"/>
+      <c r="I295" t="inlineStr"/>
       <c r="J295" t="b">
-        <v>1</v>
-      </c>
-      <c r="K295" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K295" t="n">
+        <v>-43.13</v>
+      </c>
       <c r="L295" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="M295" t="inlineStr">
         <is>
-          <t>2026-S35</t>
+          <t>2026-S42</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Cedro Kids</t>
+          <t>Delta Sports</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -17094,27 +17106,27 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>2026-09-30T23:05:37.510801+00:00</t>
+          <t>2026-08-19T02:04:08.877497+00:00</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>2026-10-01T07:10:56.849290+00:00</t>
+          <t>2026-08-19T11:36:43.537712+00:00</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>2026-10-01T19:31:49.038306+00:00</t>
+          <t>2026-08-20T02:10:47.718408+00:00</t>
         </is>
       </c>
       <c r="G296" t="n">
-        <v>8.09</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="H296" t="n">
-        <v>12.35</v>
+        <v>14.57</v>
       </c>
       <c r="I296" t="n">
-        <v>20.44</v>
+        <v>24.11</v>
       </c>
       <c r="J296" t="b">
         <v>1</v>
@@ -17122,12 +17134,12 @@
       <c r="K296" t="inlineStr"/>
       <c r="L296" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="M296" t="inlineStr">
         <is>
-          <t>2026-S40</t>
+          <t>2026-S34</t>
         </is>
       </c>
     </row>
@@ -17222,7 +17234,7 @@
         <v>0</v>
       </c>
       <c r="K298" t="n">
-        <v>-4.28</v>
+        <v>19.71</v>
       </c>
       <c r="L298" t="inlineStr">
         <is>
@@ -17656,7 +17668,7 @@
         <v>0</v>
       </c>
       <c r="K306" t="n">
-        <v>-47.21</v>
+        <v>-23.23</v>
       </c>
       <c r="L306" t="inlineStr">
         <is>
@@ -17980,7 +17992,7 @@
         <v>0</v>
       </c>
       <c r="K312" t="n">
-        <v>1344.55</v>
+        <v>1368.54</v>
       </c>
       <c r="L312" t="inlineStr">
         <is>
@@ -18029,7 +18041,7 @@
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>27.85</v>
+        <v>51.83</v>
       </c>
       <c r="L313" t="inlineStr">
         <is>
@@ -18055,198 +18067,198 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Associado</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>2026-09-09T04:38:28.762292+00:00</t>
+          <t>2026-10-18T18:21:40.554627+00:00</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>2026-09-11T10:08:31.535489+00:00</t>
-        </is>
-      </c>
-      <c r="F314" t="inlineStr">
-        <is>
-          <t>2026-09-15T08:50:48.456109+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-19T08:58:32.107455+00:00</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr"/>
       <c r="G314" t="n">
-        <v>53.5</v>
-      </c>
-      <c r="H314" t="n">
-        <v>94.7</v>
-      </c>
-      <c r="I314" t="n">
-        <v>148.21</v>
-      </c>
+        <v>14.61</v>
+      </c>
+      <c r="H314" t="inlineStr"/>
+      <c r="I314" t="inlineStr"/>
       <c r="J314" t="b">
-        <v>1</v>
-      </c>
-      <c r="K314" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K314" t="n">
+        <v>-79.06</v>
+      </c>
       <c r="L314" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="M314" t="inlineStr">
         <is>
-          <t>2026-S37</t>
+          <t>2026-S42</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Cedro Kids</t>
+          <t>Fluxo Denim</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>PO-10464</t>
+          <t>PO-10465</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Em avaliação</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>2026-09-10T17:16:09.095754+00:00</t>
+          <t>2026-08-18T20:42:52.634346+00:00</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>2026-09-11T12:43:58.441650+00:00</t>
-        </is>
-      </c>
-      <c r="F315" t="inlineStr"/>
+          <t>2026-08-20T14:27:28.706475+00:00</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>2026-08-24T15:23:27.948638+00:00</t>
+        </is>
+      </c>
       <c r="G315" t="n">
-        <v>19.46</v>
-      </c>
-      <c r="H315" t="inlineStr"/>
-      <c r="I315" t="inlineStr"/>
+        <v>41.74</v>
+      </c>
+      <c r="H315" t="n">
+        <v>96.93000000000001</v>
+      </c>
+      <c r="I315" t="n">
+        <v>138.68</v>
+      </c>
       <c r="J315" t="b">
-        <v>0</v>
-      </c>
-      <c r="K315" t="n">
-        <v>810.05</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K315" t="inlineStr"/>
       <c r="L315" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="M315" t="inlineStr">
         <is>
-          <t>2026-S37</t>
+          <t>2026-S34</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Bravo Casa</t>
+          <t>Eterna Beleza</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>PO-10465</t>
+          <t>PO-10466</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Associado</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>2026-10-03T05:50:17.284863+00:00</t>
+          <t>2026-08-25T18:47:47.606509+00:00</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>2026-10-04T10:34:24.997077+00:00</t>
-        </is>
-      </c>
-      <c r="F316" t="inlineStr"/>
+          <t>2026-08-27T01:13:05.052293+00:00</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>2026-08-29T15:33:53.862577+00:00</t>
+        </is>
+      </c>
       <c r="G316" t="n">
-        <v>28.74</v>
-      </c>
-      <c r="H316" t="inlineStr"/>
-      <c r="I316" t="inlineStr"/>
+        <v>30.42</v>
+      </c>
+      <c r="H316" t="n">
+        <v>62.35</v>
+      </c>
+      <c r="I316" t="n">
+        <v>92.77</v>
+      </c>
       <c r="J316" t="b">
-        <v>0</v>
-      </c>
-      <c r="K316" t="n">
-        <v>269.48</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K316" t="inlineStr"/>
       <c r="L316" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="M316" t="inlineStr">
         <is>
-          <t>2026-S40</t>
+          <t>2026-S35</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Delta Sports</t>
+          <t>Alpha Moda</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>PO-10466</t>
+          <t>PO-10467</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Em avaliação</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>2026-08-31T20:52:16.144491+00:00</t>
+          <t>2026-09-13T07:19:41.643302+00:00</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>2026-09-02T08:25:46.933379+00:00</t>
-        </is>
-      </c>
-      <c r="F317" t="inlineStr">
-        <is>
-          <t>2026-09-07T06:25:58.665124+00:00</t>
-        </is>
-      </c>
+          <t>2026-09-13T12:44:32.693349+00:00</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr"/>
       <c r="G317" t="n">
-        <v>35.56</v>
-      </c>
-      <c r="H317" t="n">
-        <v>118</v>
-      </c>
-      <c r="I317" t="n">
-        <v>153.56</v>
-      </c>
+        <v>5.41</v>
+      </c>
+      <c r="H317" t="inlineStr"/>
+      <c r="I317" t="inlineStr"/>
       <c r="J317" t="b">
-        <v>1</v>
-      </c>
-      <c r="K317" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K317" t="n">
+        <v>771.98</v>
+      </c>
       <c r="L317" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="M317" t="inlineStr">
         <is>
-          <t>2026-S36</t>
+          <t>2026-S37</t>
         </is>
       </c>
     </row>
@@ -18258,7 +18270,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>PO-10467</t>
+          <t>PO-10468</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -18313,7 +18325,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>PO-10470</t>
+          <t>PO-10471</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -18368,7 +18380,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>PO-10473</t>
+          <t>PO-10474</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -18423,7 +18435,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>PO-10474</t>
+          <t>PO-10475</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -18478,7 +18490,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>PO-10476</t>
+          <t>PO-10477</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -18533,7 +18545,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>PO-10477</t>
+          <t>PO-10478</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -18588,7 +18600,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>PO-10478</t>
+          <t>PO-10479</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -18643,7 +18655,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>PO-10480</t>
+          <t>PO-10481</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -18671,7 +18683,7 @@
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>854.35</v>
+        <v>878.34</v>
       </c>
       <c r="L325" t="inlineStr">
         <is>
@@ -18692,7 +18704,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>PO-10481</t>
+          <t>PO-10482</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -18747,7 +18759,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>PO-10483</t>
+          <t>PO-10484</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -18802,7 +18814,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>PO-10487</t>
+          <t>PO-10488</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -18857,7 +18869,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>PO-10488</t>
+          <t>PO-10489</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -18885,7 +18897,7 @@
         <v>0</v>
       </c>
       <c r="K329" t="n">
-        <v>441.93</v>
+        <v>465.92</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -18906,7 +18918,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>PO-10489</t>
+          <t>PO-10490</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -18934,7 +18946,7 @@
         <v>0</v>
       </c>
       <c r="K330" t="n">
-        <v>533.71</v>
+        <v>557.6900000000001</v>
       </c>
       <c r="L330" t="inlineStr">
         <is>
@@ -18955,7 +18967,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>PO-10490</t>
+          <t>PO-10491</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -19010,7 +19022,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>PO-10491</t>
+          <t>PO-10492</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -19038,7 +19050,7 @@
         <v>0</v>
       </c>
       <c r="K332" t="n">
-        <v>1183.47</v>
+        <v>1207.46</v>
       </c>
       <c r="L332" t="inlineStr">
         <is>
@@ -19059,7 +19071,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>PO-10492</t>
+          <t>PO-10493</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -19087,7 +19099,7 @@
         <v>0</v>
       </c>
       <c r="K333" t="n">
-        <v>-40.55</v>
+        <v>-16.57</v>
       </c>
       <c r="L333" t="inlineStr">
         <is>
@@ -19108,50 +19120,44 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>PO-10493</t>
+          <t>PO-10494</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Em avaliação</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>2026-08-19T18:27:37.821516+00:00</t>
+          <t>2026-10-20T15:15:50.765955+00:00</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>2026-08-23T05:06:12.426176+00:00</t>
-        </is>
-      </c>
-      <c r="F334" t="inlineStr">
-        <is>
-          <t>2026-08-28T22:05:28.981580+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-24T01:54:25.370615+00:00</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr"/>
       <c r="G334" t="n">
         <v>82.64</v>
       </c>
-      <c r="H334" t="n">
-        <v>136.99</v>
-      </c>
-      <c r="I334" t="n">
-        <v>219.63</v>
-      </c>
+      <c r="H334" t="inlineStr"/>
+      <c r="I334" t="inlineStr"/>
       <c r="J334" t="b">
-        <v>1</v>
-      </c>
-      <c r="K334" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K334" t="n">
+        <v>-123.96</v>
+      </c>
       <c r="L334" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="M334" t="inlineStr">
         <is>
-          <t>2026-S34</t>
+          <t>2026-S43</t>
         </is>
       </c>
     </row>
@@ -19163,7 +19169,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>PO-10494</t>
+          <t>PO-10495</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -19218,7 +19224,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>PO-10497</t>
+          <t>PO-10498</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -19273,7 +19279,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>PO-10499</t>
+          <t>PO-10500</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -19301,7 +19307,7 @@
         <v>0</v>
       </c>
       <c r="K337" t="n">
-        <v>148.99</v>
+        <v>172.97</v>
       </c>
       <c r="L337" t="inlineStr">
         <is>
@@ -19322,7 +19328,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>PO-10500</t>
+          <t>PO-10501</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -19377,7 +19383,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>PO-10504</t>
+          <t>PO-10505</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -19432,7 +19438,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>PO-10505</t>
+          <t>PO-10506</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -19460,7 +19466,7 @@
         <v>0</v>
       </c>
       <c r="K340" t="n">
-        <v>-87.11</v>
+        <v>-63.12</v>
       </c>
       <c r="L340" t="inlineStr">
         <is>
@@ -19481,7 +19487,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>PO-10506</t>
+          <t>PO-10507</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -19509,7 +19515,7 @@
         <v>0</v>
       </c>
       <c r="K341" t="n">
-        <v>-76.66</v>
+        <v>-52.67</v>
       </c>
       <c r="L341" t="inlineStr">
         <is>
@@ -19530,7 +19536,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>PO-10507</t>
+          <t>PO-10508</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -19585,7 +19591,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>PO-10508</t>
+          <t>PO-10509</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -19640,7 +19646,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>PO-10510</t>
+          <t>PO-10511</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -19695,7 +19701,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>PO-10511</t>
+          <t>PO-10512</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -19750,7 +19756,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>PO-10512</t>
+          <t>PO-10513</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -19805,7 +19811,7 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>PO-10516</t>
+          <t>PO-10517</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -19860,12 +19866,12 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>PO-10518</t>
+          <t>PO-10519</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Associado</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
@@ -19878,18 +19884,24 @@
           <t>2026-10-10T04:23:28.455671+00:00</t>
         </is>
       </c>
-      <c r="F348" t="inlineStr"/>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>2026-10-15T08:31:19.903061+00:00</t>
+        </is>
+      </c>
       <c r="G348" t="n">
         <v>32.96</v>
       </c>
-      <c r="H348" t="inlineStr"/>
-      <c r="I348" t="inlineStr"/>
+      <c r="H348" t="n">
+        <v>124.13</v>
+      </c>
+      <c r="I348" t="n">
+        <v>157.09</v>
+      </c>
       <c r="J348" t="b">
-        <v>0</v>
-      </c>
-      <c r="K348" t="n">
-        <v>135.89</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K348" t="inlineStr"/>
       <c r="L348" t="inlineStr">
         <is>
           <t>2026-10</t>
@@ -19909,7 +19921,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>PO-10519</t>
+          <t>PO-10520</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -19964,7 +19976,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>PO-10520</t>
+          <t>PO-10521</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -20019,7 +20031,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>PO-10521</t>
+          <t>PO-10522</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -20047,7 +20059,7 @@
         <v>0</v>
       </c>
       <c r="K351" t="n">
-        <v>1380.87</v>
+        <v>1404.85</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -20068,7 +20080,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>PO-10522</t>
+          <t>PO-10523</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -20096,7 +20108,7 @@
         <v>0</v>
       </c>
       <c r="K352" t="n">
-        <v>-49.26</v>
+        <v>-25.27</v>
       </c>
       <c r="L352" t="inlineStr">
         <is>
@@ -20117,7 +20129,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>PO-10523</t>
+          <t>PO-10524</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -20145,7 +20157,7 @@
         <v>0</v>
       </c>
       <c r="K353" t="n">
-        <v>-38.63</v>
+        <v>-14.64</v>
       </c>
       <c r="L353" t="inlineStr">
         <is>
@@ -20166,7 +20178,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>PO-10527</t>
+          <t>PO-10528</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -20221,7 +20233,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>PO-10529</t>
+          <t>PO-10530</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -20276,7 +20288,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>PO-10531</t>
+          <t>PO-10532</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -20331,7 +20343,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>PO-10532</t>
+          <t>PO-10533</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -20359,7 +20371,7 @@
         <v>0</v>
       </c>
       <c r="K357" t="n">
-        <v>1375.58</v>
+        <v>1399.57</v>
       </c>
       <c r="L357" t="inlineStr">
         <is>
@@ -20380,7 +20392,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>PO-10534</t>
+          <t>PO-10535</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -20408,7 +20420,7 @@
         <v>0</v>
       </c>
       <c r="K358" t="n">
-        <v>1562.02</v>
+        <v>1586</v>
       </c>
       <c r="L358" t="inlineStr">
         <is>
@@ -20429,7 +20441,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>PO-10537</t>
+          <t>PO-10538</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -20484,7 +20496,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>PO-10538</t>
+          <t>PO-10539</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -20512,7 +20524,7 @@
         <v>0</v>
       </c>
       <c r="K360" t="n">
-        <v>1415.78</v>
+        <v>1439.77</v>
       </c>
       <c r="L360" t="inlineStr">
         <is>
@@ -20533,7 +20545,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>PO-10539</t>
+          <t>PO-10540</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -20588,7 +20600,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>PO-10540</t>
+          <t>PO-10541</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -20643,7 +20655,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>PO-10541</t>
+          <t>PO-10542</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -20698,7 +20710,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>PO-10542</t>
+          <t>PO-10543</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -20726,7 +20738,7 @@
         <v>0</v>
       </c>
       <c r="K364" t="n">
-        <v>897.65</v>
+        <v>921.64</v>
       </c>
       <c r="L364" t="inlineStr">
         <is>
@@ -20747,7 +20759,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>PO-10544</t>
+          <t>PO-10545</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -20802,7 +20814,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>PO-10545</t>
+          <t>PO-10546</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -20857,7 +20869,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>PO-10547</t>
+          <t>PO-10548</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -20885,7 +20897,7 @@
         <v>0</v>
       </c>
       <c r="K367" t="n">
-        <v>-27.67</v>
+        <v>-3.68</v>
       </c>
       <c r="L367" t="inlineStr">
         <is>
@@ -20906,7 +20918,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>PO-10548</t>
+          <t>PO-10549</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -20961,7 +20973,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>PO-10549</t>
+          <t>PO-10550</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -21016,7 +21028,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>PO-10550</t>
+          <t>PO-10551</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -21071,7 +21083,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>PO-10551</t>
+          <t>PO-10552</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -21099,7 +21111,7 @@
         <v>0</v>
       </c>
       <c r="K371" t="n">
-        <v>690.25</v>
+        <v>714.23</v>
       </c>
       <c r="L371" t="inlineStr">
         <is>
@@ -21120,7 +21132,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>PO-10552</t>
+          <t>PO-10553</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -21175,7 +21187,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>PO-10554</t>
+          <t>PO-10555</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -21230,7 +21242,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>PO-10556</t>
+          <t>PO-10557</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -21285,7 +21297,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>PO-10557</t>
+          <t>PO-10558</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -21313,7 +21325,7 @@
         <v>0</v>
       </c>
       <c r="K375" t="n">
-        <v>32.27</v>
+        <v>56.26</v>
       </c>
       <c r="L375" t="inlineStr">
         <is>
@@ -21334,7 +21346,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>PO-10558</t>
+          <t>PO-10559</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -21389,7 +21401,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>PO-10559</t>
+          <t>PO-10560</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -21444,7 +21456,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>PO-10563</t>
+          <t>PO-10564</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
@@ -21499,7 +21511,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>PO-10564</t>
+          <t>PO-10565</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
@@ -21554,7 +21566,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>PO-10566</t>
+          <t>PO-10567</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
@@ -21609,7 +21621,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>PO-10567</t>
+          <t>PO-10568</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
@@ -21664,7 +21676,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>PO-10571</t>
+          <t>PO-10572</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
@@ -21719,7 +21731,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>PO-10572</t>
+          <t>PO-10573</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
@@ -21747,7 +21759,7 @@
         <v>0</v>
       </c>
       <c r="K383" t="n">
-        <v>1187.15</v>
+        <v>1211.13</v>
       </c>
       <c r="L383" t="inlineStr">
         <is>
@@ -21768,7 +21780,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>PO-10573</t>
+          <t>PO-10574</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
@@ -21823,7 +21835,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>PO-10574</t>
+          <t>PO-10575</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
@@ -21878,7 +21890,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>PO-10578</t>
+          <t>PO-10579</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -21933,7 +21945,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>PO-10580</t>
+          <t>PO-10581</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
@@ -21961,7 +21973,7 @@
         <v>0</v>
       </c>
       <c r="K387" t="n">
-        <v>814.9400000000001</v>
+        <v>838.9299999999999</v>
       </c>
       <c r="L387" t="inlineStr">
         <is>
@@ -21982,7 +21994,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>PO-10581</t>
+          <t>PO-10582</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
@@ -22010,7 +22022,7 @@
         <v>0</v>
       </c>
       <c r="K388" t="n">
-        <v>945.54</v>
+        <v>969.53</v>
       </c>
       <c r="L388" t="inlineStr">
         <is>
@@ -22031,7 +22043,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>PO-10582</t>
+          <t>PO-10583</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
@@ -22086,7 +22098,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>PO-10585</t>
+          <t>PO-10586</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
@@ -22141,7 +22153,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>PO-10586</t>
+          <t>PO-10587</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
@@ -22196,7 +22208,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>PO-10589</t>
+          <t>PO-10590</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
@@ -22251,7 +22263,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>PO-10590</t>
+          <t>PO-10591</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
@@ -22306,7 +22318,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>PO-10593</t>
+          <t>PO-10594</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
@@ -22334,7 +22346,7 @@
         <v>0</v>
       </c>
       <c r="K394" t="n">
-        <v>419.01</v>
+        <v>443</v>
       </c>
       <c r="L394" t="inlineStr">
         <is>
@@ -22355,7 +22367,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>PO-10594</t>
+          <t>PO-10595</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
@@ -22383,7 +22395,7 @@
         <v>0</v>
       </c>
       <c r="K395" t="n">
-        <v>-65.63</v>
+        <v>-41.65</v>
       </c>
       <c r="L395" t="inlineStr">
         <is>
@@ -22404,7 +22416,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>PO-10595</t>
+          <t>PO-10596</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
@@ -22448,55 +22460,6 @@
       <c r="M396" t="inlineStr">
         <is>
           <t>2026-S38</t>
-        </is>
-      </c>
-    </row>
-    <row r="397">
-      <c r="A397" t="inlineStr">
-        <is>
-          <t>Bravo Casa</t>
-        </is>
-      </c>
-      <c r="B397" t="inlineStr">
-        <is>
-          <t>PO-10599</t>
-        </is>
-      </c>
-      <c r="C397" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="D397" t="inlineStr">
-        <is>
-          <t>2026-09-02T23:40:14.276060+00:00</t>
-        </is>
-      </c>
-      <c r="E397" t="inlineStr">
-        <is>
-          <t>2026-09-03T14:16:36.045318+00:00</t>
-        </is>
-      </c>
-      <c r="F397" t="inlineStr"/>
-      <c r="G397" t="n">
-        <v>14.61</v>
-      </c>
-      <c r="H397" t="inlineStr"/>
-      <c r="I397" t="inlineStr"/>
-      <c r="J397" t="b">
-        <v>0</v>
-      </c>
-      <c r="K397" t="n">
-        <v>995.65</v>
-      </c>
-      <c r="L397" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="M397" t="inlineStr">
-        <is>
-          <t>2026-S36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza painel (2026-10-16 11:18 UTC)
</commit_message>
<xml_diff>
--- a/dados/status_atual.xlsx
+++ b/dados/status_atual.xlsx
@@ -452,7 +452,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>95.90000000000001</v>
+        <v>96</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -463,7 +463,7 @@
         <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>262</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3">
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>82.3</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -484,7 +484,7 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>295</v>
+        <v>299</v>
       </c>
     </row>
     <row r="4">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>72.8</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -505,7 +505,7 @@
         <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>316</v>
+        <v>312</v>
       </c>
     </row>
     <row r="5">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>60.4</v>
+        <v>60.6</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -526,7 +526,7 @@
         <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6">
@@ -547,7 +547,7 @@
         <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="7">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>25.2</v>
+        <v>25.6</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -568,7 +568,7 @@
         <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -644,10 +644,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F2" t="n">
         <v>2</v>
@@ -656,7 +656,7 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>96</v>
+        <v>96.09999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -676,10 +676,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E3" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F3" t="n">
         <v>2</v>
@@ -708,10 +708,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E4" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F4" t="n">
         <v>5</v>
@@ -720,7 +720,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>93.90000000000001</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5">
@@ -740,10 +740,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E5" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F5" t="n">
         <v>2</v>
@@ -752,7 +752,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>96.5</v>
+        <v>96.59999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -772,10 +772,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E6" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F6" t="n">
         <v>10</v>
@@ -784,7 +784,7 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>82.8</v>
+        <v>83.09999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -804,10 +804,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E7" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F7" t="n">
         <v>12</v>
@@ -816,7 +816,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>84.8</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8">
@@ -836,10 +836,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E8" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F8" t="n">
         <v>20</v>
@@ -848,7 +848,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>77.5</v>
+        <v>77.8</v>
       </c>
     </row>
     <row r="9">
@@ -868,10 +868,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E9" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F9" t="n">
         <v>11</v>
@@ -880,7 +880,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>84.09999999999999</v>
+        <v>84.3</v>
       </c>
     </row>
     <row r="10">
@@ -964,19 +964,19 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E12" t="n">
         <v>51</v>
       </c>
       <c r="F12" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>64.59999999999999</v>
+        <v>65.40000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -1060,10 +1060,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E15" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F15" t="n">
         <v>48</v>
@@ -1072,7 +1072,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>45.5</v>
+        <v>46.1</v>
       </c>
     </row>
     <row r="16">
@@ -1092,19 +1092,19 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E16" t="n">
         <v>49</v>
       </c>
       <c r="F16" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>46.7</v>
+        <v>46.2</v>
       </c>
     </row>
     <row r="17">
@@ -1156,19 +1156,19 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E18" t="n">
         <v>12</v>
       </c>
       <c r="F18" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>25.5</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="19">
@@ -1188,19 +1188,19 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E19" t="n">
         <v>18</v>
       </c>
       <c r="F19" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>26.9</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="20">
@@ -1220,19 +1220,19 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
       </c>
       <c r="F20" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>27.3</v>
+        <v>27.6</v>
       </c>
     </row>
     <row r="21">
@@ -1252,19 +1252,19 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E21" t="n">
         <v>12</v>
       </c>
       <c r="F21" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>21.1</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="22">
@@ -1284,19 +1284,19 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E22" t="n">
         <v>48</v>
       </c>
       <c r="F22" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>70.59999999999999</v>
+        <v>71.59999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -1316,10 +1316,10 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E23" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F23" t="n">
         <v>23</v>
@@ -1328,7 +1328,7 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>72.3</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24">
@@ -1348,10 +1348,10 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E24" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F24" t="n">
         <v>15</v>
@@ -1360,7 +1360,7 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>82.8</v>
+        <v>82.59999999999999</v>
       </c>
     </row>
     <row r="25">
@@ -1380,19 +1380,19 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E25" t="n">
         <v>51</v>
       </c>
       <c r="F25" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>65.40000000000001</v>
+        <v>66.2</v>
       </c>
     </row>
   </sheetData>
@@ -1622,7 +1622,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>1007.62</v>
+        <v>1031.63</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -1781,7 +1781,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>1118.75</v>
+        <v>1142.75</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -1830,7 +1830,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>242.96</v>
+        <v>266.96</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>45.69</v>
+        <v>69.7</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -1928,7 +1928,7 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>1497.63</v>
+        <v>1521.63</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>318.13</v>
+        <v>342.13</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -2026,7 +2026,7 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>-58.26</v>
+        <v>-34.26</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>904.09</v>
+        <v>928.09</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -2124,7 +2124,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>1261.12</v>
+        <v>1285.13</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Em avaliação</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2493,18 +2493,24 @@
           <t>2026-10-12T10:11:27.407818+00:00</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-10-16T02:47:42.147096+00:00</t>
+        </is>
+      </c>
       <c r="G21" t="n">
         <v>44.87</v>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>88.59999999999999</v>
+      </c>
+      <c r="I21" t="n">
+        <v>133.47</v>
+      </c>
       <c r="J21" t="b">
-        <v>0</v>
-      </c>
-      <c r="K21" t="n">
-        <v>117.98</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>2026-10</t>
@@ -2717,7 +2723,7 @@
         <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>354.03</v>
+        <v>378.03</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -2986,7 +2992,7 @@
         <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>1701.4</v>
+        <v>1725.4</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -3420,7 +3426,7 @@
         <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>-7.93</v>
+        <v>16.07</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -3524,7 +3530,7 @@
         <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>20.14</v>
+        <v>44.15</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -3573,7 +3579,7 @@
         <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>441.61</v>
+        <v>465.61</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -3764,22 +3770,22 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Em avaliação</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2026-09-19T09:20:01.939484+00:00</t>
+          <t>2026-10-18T20:04:34.183434+00:00</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-09-19T19:55:30.753710+00:00</t>
+          <t>2026-10-21T20:08:35.710620+00:00</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="n">
-        <v>10.59</v>
+        <v>72.06999999999999</v>
       </c>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
@@ -3787,16 +3793,16 @@
         <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>625.97</v>
+        <v>-56.77</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>2026-S38</t>
+          <t>2026-S42</t>
         </is>
       </c>
     </row>
@@ -3808,7 +3814,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PO-10078</t>
+          <t>PO-10079</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3863,7 +3869,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PO-10080</t>
+          <t>PO-10081</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3918,7 +3924,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PO-10081</t>
+          <t>PO-10082</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3973,7 +3979,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PO-10083</t>
+          <t>PO-10084</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -4028,7 +4034,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PO-10084</t>
+          <t>PO-10085</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -4083,7 +4089,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PO-10085</t>
+          <t>PO-10086</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -4111,7 +4117,7 @@
         <v>0</v>
       </c>
       <c r="K51" t="n">
-        <v>1074.6</v>
+        <v>1098.6</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -4132,7 +4138,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PO-10086</t>
+          <t>PO-10087</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -4187,7 +4193,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PO-10087</t>
+          <t>PO-10088</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -4215,7 +4221,7 @@
         <v>0</v>
       </c>
       <c r="K53" t="n">
-        <v>1108.92</v>
+        <v>1132.92</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -4236,7 +4242,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PO-10088</t>
+          <t>PO-10089</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -4291,7 +4297,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PO-10089</t>
+          <t>PO-10090</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -4319,7 +4325,7 @@
         <v>0</v>
       </c>
       <c r="K55" t="n">
-        <v>-22.48</v>
+        <v>1.53</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
@@ -4340,7 +4346,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PO-10090</t>
+          <t>PO-10091</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -4390,7 +4396,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Eterna Beleza</t>
+          <t>Bravo Casa</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -4400,22 +4406,22 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Em avaliação</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2026-10-17T22:10:39.562579+00:00</t>
+          <t>2026-10-19T05:07:32.546408+00:00</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-10-18T11:36:47.720708+00:00</t>
+          <t>2026-10-19T15:10:19.810830+00:00</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="n">
-        <v>13.44</v>
+        <v>10.05</v>
       </c>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr"/>
@@ -4423,7 +4429,7 @@
         <v>0</v>
       </c>
       <c r="K57" t="n">
-        <v>-58.87</v>
+        <v>-65.81999999999999</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
@@ -4432,14 +4438,14 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>2026-S42</t>
+          <t>2026-S43</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Fluxo Denim</t>
+          <t>Alpha Moda</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -4449,31 +4455,37 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Associado</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2026-08-06T11:45:05.928880+00:00</t>
+          <t>2026-08-31T05:37:58.813763+00:00</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2026-08-07T23:12:39.210253+00:00</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
+          <t>2026-08-31T21:00:15.569141+00:00</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2026-09-03T00:32:29.255896+00:00</t>
+        </is>
+      </c>
       <c r="G58" t="n">
-        <v>35.46</v>
-      </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
+        <v>15.37</v>
+      </c>
+      <c r="H58" t="n">
+        <v>51.54</v>
+      </c>
+      <c r="I58" t="n">
+        <v>66.91</v>
+      </c>
       <c r="J58" t="b">
-        <v>0</v>
-      </c>
-      <c r="K58" t="n">
-        <v>1679.55</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
           <t>2026-08</t>
@@ -4481,7 +4493,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>2026-S32</t>
+          <t>2026-S36</t>
         </is>
       </c>
     </row>
@@ -4686,7 +4698,7 @@
         <v>0</v>
       </c>
       <c r="K62" t="n">
-        <v>787.03</v>
+        <v>811.03</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -4827,12 +4839,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2026-10-15T03:41:22.502957+00:00</t>
+          <t>2026-10-18T09:41:22.502957+00:00</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2026-10-18T01:33:13.194543+00:00</t>
+          <t>2026-10-21T07:33:13.194543+00:00</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
@@ -4845,7 +4857,7 @@
         <v>0</v>
       </c>
       <c r="K65" t="n">
-        <v>7.62</v>
+        <v>-46.38</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
@@ -4894,7 +4906,7 @@
         <v>0</v>
       </c>
       <c r="K66" t="n">
-        <v>907.01</v>
+        <v>931.01</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
@@ -4943,7 +4955,7 @@
         <v>0</v>
       </c>
       <c r="K67" t="n">
-        <v>182.79</v>
+        <v>206.79</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
@@ -5047,7 +5059,7 @@
         <v>0</v>
       </c>
       <c r="K69" t="n">
-        <v>55.77</v>
+        <v>79.78</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -5348,7 +5360,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -5361,18 +5373,24 @@
           <t>2026-10-15T02:08:30.014001+00:00</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>2026-10-16T02:18:06.920590+00:00</t>
+        </is>
+      </c>
       <c r="G75" t="n">
         <v>62.45</v>
       </c>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
+      <c r="H75" t="n">
+        <v>24.16</v>
+      </c>
+      <c r="I75" t="n">
+        <v>86.61</v>
+      </c>
       <c r="J75" t="b">
-        <v>0</v>
-      </c>
-      <c r="K75" t="n">
-        <v>71.61</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
           <t>2026-10</t>
@@ -5695,7 +5713,7 @@
         <v>0</v>
       </c>
       <c r="K81" t="n">
-        <v>1526.91</v>
+        <v>1550.91</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
@@ -5964,7 +5982,7 @@
         <v>0</v>
       </c>
       <c r="K86" t="n">
-        <v>38.23</v>
+        <v>62.23</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -6270,12 +6288,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>2026-10-17T04:32:58.761059+00:00</t>
+          <t>2026-10-17T22:25:00.168390+00:00</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>2026-10-17T17:06:53.316047+00:00</t>
+          <t>2026-10-18T10:58:54.723378+00:00</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -6288,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="K92" t="n">
-        <v>-41.24</v>
+        <v>-35.11</v>
       </c>
       <c r="L92" t="inlineStr">
         <is>
@@ -6337,7 +6355,7 @@
         <v>0</v>
       </c>
       <c r="K93" t="n">
-        <v>1468.88</v>
+        <v>1492.88</v>
       </c>
       <c r="L93" t="inlineStr">
         <is>
@@ -6386,7 +6404,7 @@
         <v>0</v>
       </c>
       <c r="K94" t="n">
-        <v>1120.29</v>
+        <v>1144.29</v>
       </c>
       <c r="L94" t="inlineStr">
         <is>
@@ -6600,7 +6618,7 @@
         <v>0</v>
       </c>
       <c r="K98" t="n">
-        <v>215.7</v>
+        <v>239.7</v>
       </c>
       <c r="L98" t="inlineStr">
         <is>
@@ -7034,7 +7052,7 @@
         <v>0</v>
       </c>
       <c r="K106" t="n">
-        <v>787.09</v>
+        <v>811.09</v>
       </c>
       <c r="L106" t="inlineStr">
         <is>
@@ -7248,7 +7266,7 @@
         <v>0</v>
       </c>
       <c r="K110" t="n">
-        <v>272.16</v>
+        <v>296.16</v>
       </c>
       <c r="L110" t="inlineStr">
         <is>
@@ -7682,7 +7700,7 @@
         <v>0</v>
       </c>
       <c r="K118" t="n">
-        <v>54.89</v>
+        <v>78.89</v>
       </c>
       <c r="L118" t="inlineStr">
         <is>
@@ -8006,7 +8024,7 @@
         <v>0</v>
       </c>
       <c r="K124" t="n">
-        <v>1097.02</v>
+        <v>1121.02</v>
       </c>
       <c r="L124" t="inlineStr">
         <is>
@@ -8330,7 +8348,7 @@
         <v>0</v>
       </c>
       <c r="K130" t="n">
-        <v>1518.59</v>
+        <v>1542.6</v>
       </c>
       <c r="L130" t="inlineStr">
         <is>
@@ -8379,7 +8397,7 @@
         <v>0</v>
       </c>
       <c r="K131" t="n">
-        <v>336.79</v>
+        <v>360.79</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
@@ -8428,7 +8446,7 @@
         <v>0</v>
       </c>
       <c r="K132" t="n">
-        <v>-77.68000000000001</v>
+        <v>-53.68</v>
       </c>
       <c r="L132" t="inlineStr">
         <is>
@@ -8697,7 +8715,7 @@
         <v>0</v>
       </c>
       <c r="K137" t="n">
-        <v>1199.12</v>
+        <v>1223.12</v>
       </c>
       <c r="L137" t="inlineStr">
         <is>
@@ -8746,7 +8764,7 @@
         <v>0</v>
       </c>
       <c r="K138" t="n">
-        <v>1692.56</v>
+        <v>1716.56</v>
       </c>
       <c r="L138" t="inlineStr">
         <is>
@@ -9125,7 +9143,7 @@
         <v>0</v>
       </c>
       <c r="K145" t="n">
-        <v>298.19</v>
+        <v>322.19</v>
       </c>
       <c r="L145" t="inlineStr">
         <is>
@@ -9339,7 +9357,7 @@
         <v>0</v>
       </c>
       <c r="K149" t="n">
-        <v>25.72</v>
+        <v>49.72</v>
       </c>
       <c r="L149" t="inlineStr">
         <is>
@@ -9585,45 +9603,39 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Associado</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>2026-09-10T11:39:00.739162+00:00</t>
+          <t>2026-10-19T04:54:40.480553+00:00</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>2026-09-11T10:41:21.171244+00:00</t>
-        </is>
-      </c>
-      <c r="F154" t="inlineStr">
-        <is>
-          <t>2026-09-12T09:13:36.713937+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-20T03:57:00.912635+00:00</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr"/>
       <c r="G154" t="n">
         <v>23.04</v>
       </c>
-      <c r="H154" t="n">
-        <v>22.54</v>
-      </c>
-      <c r="I154" t="n">
-        <v>45.58</v>
-      </c>
+      <c r="H154" t="inlineStr"/>
+      <c r="I154" t="inlineStr"/>
       <c r="J154" t="b">
-        <v>1</v>
-      </c>
-      <c r="K154" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K154" t="n">
+        <v>-65.59999999999999</v>
+      </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>2026-S37</t>
+          <t>2026-S43</t>
         </is>
       </c>
     </row>
@@ -9773,7 +9785,7 @@
         <v>0</v>
       </c>
       <c r="K157" t="n">
-        <v>617.9400000000001</v>
+        <v>641.9400000000001</v>
       </c>
       <c r="L157" t="inlineStr">
         <is>
@@ -9877,7 +9889,7 @@
         <v>0</v>
       </c>
       <c r="K159" t="n">
-        <v>405.86</v>
+        <v>429.87</v>
       </c>
       <c r="L159" t="inlineStr">
         <is>
@@ -9981,7 +9993,7 @@
         <v>0</v>
       </c>
       <c r="K161" t="n">
-        <v>1285.59</v>
+        <v>1309.6</v>
       </c>
       <c r="L161" t="inlineStr">
         <is>
@@ -10085,7 +10097,7 @@
         <v>0</v>
       </c>
       <c r="K163" t="n">
-        <v>591.49</v>
+        <v>615.5</v>
       </c>
       <c r="L163" t="inlineStr">
         <is>
@@ -10189,7 +10201,7 @@
         <v>0</v>
       </c>
       <c r="K165" t="n">
-        <v>-8.98</v>
+        <v>15.03</v>
       </c>
       <c r="L165" t="inlineStr">
         <is>
@@ -10293,7 +10305,7 @@
         <v>0</v>
       </c>
       <c r="K167" t="n">
-        <v>1256.08</v>
+        <v>1280.08</v>
       </c>
       <c r="L167" t="inlineStr">
         <is>
@@ -10672,7 +10684,7 @@
         <v>0</v>
       </c>
       <c r="K174" t="n">
-        <v>1192.19</v>
+        <v>1216.19</v>
       </c>
       <c r="L174" t="inlineStr">
         <is>
@@ -11216,7 +11228,7 @@
         <v>0</v>
       </c>
       <c r="K184" t="n">
-        <v>1018.87</v>
+        <v>1042.88</v>
       </c>
       <c r="L184" t="inlineStr">
         <is>
@@ -11320,7 +11332,7 @@
         <v>0</v>
       </c>
       <c r="K186" t="n">
-        <v>9.640000000000001</v>
+        <v>33.64</v>
       </c>
       <c r="L186" t="inlineStr">
         <is>
@@ -11424,7 +11436,7 @@
         <v>0</v>
       </c>
       <c r="K188" t="n">
-        <v>149.04</v>
+        <v>173.04</v>
       </c>
       <c r="L188" t="inlineStr">
         <is>
@@ -11560,7 +11572,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Associado</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -11573,18 +11585,24 @@
           <t>2026-10-13T16:04:56.078166+00:00</t>
         </is>
       </c>
-      <c r="F191" t="inlineStr"/>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>2026-10-16T01:14:59.802480+00:00</t>
+        </is>
+      </c>
       <c r="G191" t="n">
         <v>52.04</v>
       </c>
-      <c r="H191" t="inlineStr"/>
-      <c r="I191" t="inlineStr"/>
+      <c r="H191" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="I191" t="n">
+        <v>109.2</v>
+      </c>
       <c r="J191" t="b">
-        <v>0</v>
-      </c>
-      <c r="K191" t="n">
-        <v>95.26000000000001</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K191" t="inlineStr"/>
       <c r="L191" t="inlineStr">
         <is>
           <t>2026-10</t>
@@ -11632,7 +11650,7 @@
         <v>0</v>
       </c>
       <c r="K192" t="n">
-        <v>-75.84999999999999</v>
+        <v>-51.84</v>
       </c>
       <c r="L192" t="inlineStr">
         <is>
@@ -11736,7 +11754,7 @@
         <v>0</v>
       </c>
       <c r="K194" t="n">
-        <v>68.90000000000001</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="L194" t="inlineStr">
         <is>
@@ -11840,7 +11858,7 @@
         <v>0</v>
       </c>
       <c r="K196" t="n">
-        <v>1447.06</v>
+        <v>1471.06</v>
       </c>
       <c r="L196" t="inlineStr">
         <is>
@@ -12054,7 +12072,7 @@
         <v>0</v>
       </c>
       <c r="K200" t="n">
-        <v>1766.11</v>
+        <v>1790.11</v>
       </c>
       <c r="L200" t="inlineStr">
         <is>
@@ -12103,7 +12121,7 @@
         <v>0</v>
       </c>
       <c r="K201" t="n">
-        <v>-22.46</v>
+        <v>1.55</v>
       </c>
       <c r="L201" t="inlineStr">
         <is>
@@ -12152,7 +12170,7 @@
         <v>0</v>
       </c>
       <c r="K202" t="n">
-        <v>259.31</v>
+        <v>283.32</v>
       </c>
       <c r="L202" t="inlineStr">
         <is>
@@ -12476,7 +12494,7 @@
         <v>0</v>
       </c>
       <c r="K208" t="n">
-        <v>289.66</v>
+        <v>313.66</v>
       </c>
       <c r="L208" t="inlineStr">
         <is>
@@ -12525,7 +12543,7 @@
         <v>0</v>
       </c>
       <c r="K209" t="n">
-        <v>5.28</v>
+        <v>29.28</v>
       </c>
       <c r="L209" t="inlineStr">
         <is>
@@ -12574,7 +12592,7 @@
         <v>0</v>
       </c>
       <c r="K210" t="n">
-        <v>69.92</v>
+        <v>93.92</v>
       </c>
       <c r="L210" t="inlineStr">
         <is>
@@ -12678,7 +12696,7 @@
         <v>0</v>
       </c>
       <c r="K212" t="n">
-        <v>1359.41</v>
+        <v>1383.42</v>
       </c>
       <c r="L212" t="inlineStr">
         <is>
@@ -12782,7 +12800,7 @@
         <v>0</v>
       </c>
       <c r="K214" t="n">
-        <v>28.96</v>
+        <v>52.97</v>
       </c>
       <c r="L214" t="inlineStr">
         <is>
@@ -12831,7 +12849,7 @@
         <v>0</v>
       </c>
       <c r="K215" t="n">
-        <v>1088.77</v>
+        <v>1112.77</v>
       </c>
       <c r="L215" t="inlineStr">
         <is>
@@ -13045,7 +13063,7 @@
         <v>0</v>
       </c>
       <c r="K219" t="n">
-        <v>-10.81</v>
+        <v>13.19</v>
       </c>
       <c r="L219" t="inlineStr">
         <is>
@@ -13314,7 +13332,7 @@
         <v>0</v>
       </c>
       <c r="K224" t="n">
-        <v>1478.53</v>
+        <v>1502.53</v>
       </c>
       <c r="L224" t="inlineStr">
         <is>
@@ -13418,7 +13436,7 @@
         <v>0</v>
       </c>
       <c r="K226" t="n">
-        <v>-25.9</v>
+        <v>-1.89</v>
       </c>
       <c r="L226" t="inlineStr">
         <is>
@@ -13522,7 +13540,7 @@
         <v>0</v>
       </c>
       <c r="K228" t="n">
-        <v>1599.08</v>
+        <v>1623.09</v>
       </c>
       <c r="L228" t="inlineStr">
         <is>
@@ -13571,7 +13589,7 @@
         <v>0</v>
       </c>
       <c r="K229" t="n">
-        <v>923.45</v>
+        <v>947.45</v>
       </c>
       <c r="L229" t="inlineStr">
         <is>
@@ -13730,7 +13748,7 @@
         <v>0</v>
       </c>
       <c r="K232" t="n">
-        <v>1595.99</v>
+        <v>1619.99</v>
       </c>
       <c r="L232" t="inlineStr">
         <is>
@@ -13999,7 +14017,7 @@
         <v>0</v>
       </c>
       <c r="K237" t="n">
-        <v>532.34</v>
+        <v>556.34</v>
       </c>
       <c r="L237" t="inlineStr">
         <is>
@@ -14048,7 +14066,7 @@
         <v>0</v>
       </c>
       <c r="K238" t="n">
-        <v>1644.24</v>
+        <v>1668.24</v>
       </c>
       <c r="L238" t="inlineStr">
         <is>
@@ -14097,7 +14115,7 @@
         <v>0</v>
       </c>
       <c r="K239" t="n">
-        <v>202.77</v>
+        <v>226.77</v>
       </c>
       <c r="L239" t="inlineStr">
         <is>
@@ -14256,7 +14274,7 @@
         <v>0</v>
       </c>
       <c r="K242" t="n">
-        <v>-39.1</v>
+        <v>-15.09</v>
       </c>
       <c r="L242" t="inlineStr">
         <is>
@@ -14557,7 +14575,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Em avaliação</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -14570,18 +14588,24 @@
           <t>2026-10-13T13:38:39.061234+00:00</t>
         </is>
       </c>
-      <c r="F248" t="inlineStr"/>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>2026-10-15T23:37:57.281330+00:00</t>
+        </is>
+      </c>
       <c r="G248" t="n">
         <v>5.6</v>
       </c>
-      <c r="H248" t="inlineStr"/>
-      <c r="I248" t="inlineStr"/>
+      <c r="H248" t="n">
+        <v>57.99</v>
+      </c>
+      <c r="I248" t="n">
+        <v>63.58</v>
+      </c>
       <c r="J248" t="b">
-        <v>0</v>
-      </c>
-      <c r="K248" t="n">
-        <v>51.26</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K248" t="inlineStr"/>
       <c r="L248" t="inlineStr">
         <is>
           <t>2026-10</t>
@@ -14849,7 +14873,7 @@
         <v>0</v>
       </c>
       <c r="K253" t="n">
-        <v>-74.09</v>
+        <v>-50.09</v>
       </c>
       <c r="L253" t="inlineStr">
         <is>
@@ -15228,7 +15252,7 @@
         <v>0</v>
       </c>
       <c r="K260" t="n">
-        <v>88.84</v>
+        <v>112.84</v>
       </c>
       <c r="L260" t="inlineStr">
         <is>
@@ -15277,7 +15301,7 @@
         <v>0</v>
       </c>
       <c r="K261" t="n">
-        <v>108.92</v>
+        <v>132.92</v>
       </c>
       <c r="L261" t="inlineStr">
         <is>
@@ -15546,7 +15570,7 @@
         <v>0</v>
       </c>
       <c r="K266" t="n">
-        <v>1054.93</v>
+        <v>1078.93</v>
       </c>
       <c r="L266" t="inlineStr">
         <is>
@@ -15650,7 +15674,7 @@
         <v>0</v>
       </c>
       <c r="K268" t="n">
-        <v>1723.62</v>
+        <v>1747.62</v>
       </c>
       <c r="L268" t="inlineStr">
         <is>
@@ -15754,7 +15778,7 @@
         <v>0</v>
       </c>
       <c r="K270" t="n">
-        <v>1223.54</v>
+        <v>1247.54</v>
       </c>
       <c r="L270" t="inlineStr">
         <is>
@@ -15803,7 +15827,7 @@
         <v>0</v>
       </c>
       <c r="K271" t="n">
-        <v>1694.79</v>
+        <v>1718.79</v>
       </c>
       <c r="L271" t="inlineStr">
         <is>
@@ -15852,7 +15876,7 @@
         <v>0</v>
       </c>
       <c r="K272" t="n">
-        <v>324.08</v>
+        <v>348.09</v>
       </c>
       <c r="L272" t="inlineStr">
         <is>
@@ -15901,7 +15925,7 @@
         <v>0</v>
       </c>
       <c r="K273" t="n">
-        <v>1440.49</v>
+        <v>1464.49</v>
       </c>
       <c r="L273" t="inlineStr">
         <is>
@@ -16005,7 +16029,7 @@
         <v>0</v>
       </c>
       <c r="K275" t="n">
-        <v>770.34</v>
+        <v>794.35</v>
       </c>
       <c r="L275" t="inlineStr">
         <is>
@@ -16054,7 +16078,7 @@
         <v>0</v>
       </c>
       <c r="K276" t="n">
-        <v>140.92</v>
+        <v>164.92</v>
       </c>
       <c r="L276" t="inlineStr">
         <is>
@@ -16378,7 +16402,7 @@
         <v>0</v>
       </c>
       <c r="K282" t="n">
-        <v>1229.31</v>
+        <v>1253.32</v>
       </c>
       <c r="L282" t="inlineStr">
         <is>
@@ -16867,7 +16891,7 @@
         <v>0</v>
       </c>
       <c r="K291" t="n">
-        <v>36.18</v>
+        <v>60.19</v>
       </c>
       <c r="L291" t="inlineStr">
         <is>
@@ -16916,7 +16940,7 @@
         <v>0</v>
       </c>
       <c r="K292" t="n">
-        <v>904.53</v>
+        <v>928.54</v>
       </c>
       <c r="L292" t="inlineStr">
         <is>
@@ -17075,7 +17099,7 @@
         <v>0</v>
       </c>
       <c r="K295" t="n">
-        <v>-43.13</v>
+        <v>-19.13</v>
       </c>
       <c r="L295" t="inlineStr">
         <is>
@@ -17234,7 +17258,7 @@
         <v>0</v>
       </c>
       <c r="K298" t="n">
-        <v>19.71</v>
+        <v>43.71</v>
       </c>
       <c r="L298" t="inlineStr">
         <is>
@@ -17668,7 +17692,7 @@
         <v>0</v>
       </c>
       <c r="K306" t="n">
-        <v>-23.23</v>
+        <v>0.78</v>
       </c>
       <c r="L306" t="inlineStr">
         <is>
@@ -17992,7 +18016,7 @@
         <v>0</v>
       </c>
       <c r="K312" t="n">
-        <v>1368.54</v>
+        <v>1392.54</v>
       </c>
       <c r="L312" t="inlineStr">
         <is>
@@ -18041,7 +18065,7 @@
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>51.83</v>
+        <v>75.84</v>
       </c>
       <c r="L313" t="inlineStr">
         <is>
@@ -18090,7 +18114,7 @@
         <v>0</v>
       </c>
       <c r="K314" t="n">
-        <v>-79.06</v>
+        <v>-55.05</v>
       </c>
       <c r="L314" t="inlineStr">
         <is>
@@ -18249,7 +18273,7 @@
         <v>0</v>
       </c>
       <c r="K317" t="n">
-        <v>771.98</v>
+        <v>795.98</v>
       </c>
       <c r="L317" t="inlineStr">
         <is>
@@ -18683,7 +18707,7 @@
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>878.34</v>
+        <v>902.34</v>
       </c>
       <c r="L325" t="inlineStr">
         <is>
@@ -18897,7 +18921,7 @@
         <v>0</v>
       </c>
       <c r="K329" t="n">
-        <v>465.92</v>
+        <v>489.92</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -18946,7 +18970,7 @@
         <v>0</v>
       </c>
       <c r="K330" t="n">
-        <v>557.6900000000001</v>
+        <v>581.7</v>
       </c>
       <c r="L330" t="inlineStr">
         <is>
@@ -19050,7 +19074,7 @@
         <v>0</v>
       </c>
       <c r="K332" t="n">
-        <v>1207.46</v>
+        <v>1231.46</v>
       </c>
       <c r="L332" t="inlineStr">
         <is>
@@ -19099,7 +19123,7 @@
         <v>0</v>
       </c>
       <c r="K333" t="n">
-        <v>-16.57</v>
+        <v>7.44</v>
       </c>
       <c r="L333" t="inlineStr">
         <is>
@@ -19148,7 +19172,7 @@
         <v>0</v>
       </c>
       <c r="K334" t="n">
-        <v>-123.96</v>
+        <v>-99.95999999999999</v>
       </c>
       <c r="L334" t="inlineStr">
         <is>
@@ -19307,7 +19331,7 @@
         <v>0</v>
       </c>
       <c r="K337" t="n">
-        <v>172.97</v>
+        <v>196.98</v>
       </c>
       <c r="L337" t="inlineStr">
         <is>
@@ -19466,7 +19490,7 @@
         <v>0</v>
       </c>
       <c r="K340" t="n">
-        <v>-63.12</v>
+        <v>-39.12</v>
       </c>
       <c r="L340" t="inlineStr">
         <is>
@@ -19515,7 +19539,7 @@
         <v>0</v>
       </c>
       <c r="K341" t="n">
-        <v>-52.67</v>
+        <v>-28.67</v>
       </c>
       <c r="L341" t="inlineStr">
         <is>
@@ -20059,7 +20083,7 @@
         <v>0</v>
       </c>
       <c r="K351" t="n">
-        <v>1404.85</v>
+        <v>1428.86</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -20108,7 +20132,7 @@
         <v>0</v>
       </c>
       <c r="K352" t="n">
-        <v>-25.27</v>
+        <v>-1.27</v>
       </c>
       <c r="L352" t="inlineStr">
         <is>
@@ -20157,7 +20181,7 @@
         <v>0</v>
       </c>
       <c r="K353" t="n">
-        <v>-14.64</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="L353" t="inlineStr">
         <is>
@@ -20371,7 +20395,7 @@
         <v>0</v>
       </c>
       <c r="K357" t="n">
-        <v>1399.57</v>
+        <v>1423.57</v>
       </c>
       <c r="L357" t="inlineStr">
         <is>
@@ -20420,7 +20444,7 @@
         <v>0</v>
       </c>
       <c r="K358" t="n">
-        <v>1586</v>
+        <v>1610.01</v>
       </c>
       <c r="L358" t="inlineStr">
         <is>
@@ -20524,7 +20548,7 @@
         <v>0</v>
       </c>
       <c r="K360" t="n">
-        <v>1439.77</v>
+        <v>1463.77</v>
       </c>
       <c r="L360" t="inlineStr">
         <is>
@@ -20738,7 +20762,7 @@
         <v>0</v>
       </c>
       <c r="K364" t="n">
-        <v>921.64</v>
+        <v>945.64</v>
       </c>
       <c r="L364" t="inlineStr">
         <is>
@@ -20897,7 +20921,7 @@
         <v>0</v>
       </c>
       <c r="K367" t="n">
-        <v>-3.68</v>
+        <v>20.32</v>
       </c>
       <c r="L367" t="inlineStr">
         <is>
@@ -21111,7 +21135,7 @@
         <v>0</v>
       </c>
       <c r="K371" t="n">
-        <v>714.23</v>
+        <v>738.24</v>
       </c>
       <c r="L371" t="inlineStr">
         <is>
@@ -21325,7 +21349,7 @@
         <v>0</v>
       </c>
       <c r="K375" t="n">
-        <v>56.26</v>
+        <v>80.26000000000001</v>
       </c>
       <c r="L375" t="inlineStr">
         <is>
@@ -21759,7 +21783,7 @@
         <v>0</v>
       </c>
       <c r="K383" t="n">
-        <v>1211.13</v>
+        <v>1235.14</v>
       </c>
       <c r="L383" t="inlineStr">
         <is>
@@ -21973,7 +21997,7 @@
         <v>0</v>
       </c>
       <c r="K387" t="n">
-        <v>838.9299999999999</v>
+        <v>862.9299999999999</v>
       </c>
       <c r="L387" t="inlineStr">
         <is>
@@ -22022,7 +22046,7 @@
         <v>0</v>
       </c>
       <c r="K388" t="n">
-        <v>969.53</v>
+        <v>993.53</v>
       </c>
       <c r="L388" t="inlineStr">
         <is>
@@ -22346,7 +22370,7 @@
         <v>0</v>
       </c>
       <c r="K394" t="n">
-        <v>443</v>
+        <v>467</v>
       </c>
       <c r="L394" t="inlineStr">
         <is>
@@ -22395,7 +22419,7 @@
         <v>0</v>
       </c>
       <c r="K395" t="n">
-        <v>-41.65</v>
+        <v>-17.64</v>
       </c>
       <c r="L395" t="inlineStr">
         <is>

</xml_diff>